<commit_message>
docs/lab: bổ sung rà soát SMART, phạm vi, câu hỏi ưu tiên, sơ đồ cây WBS và phương án nén lịch
- Excel: sheet NenLich (fast-tracking + dời FR09–FR10), T 75,33 -> 61,83 ngày, P(kịp hạn) ~74%
- Word: mục 2.1, 2.2, 2.9, 3.1, 4.5; nhật ký AI ghi rõ phần do Claude Code soạn

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/lab/QLDA_PharmaDash_LichDuAn.xlsx
+++ b/docs/lab/QLDA_PharmaDash_LichDuAn.xlsx
@@ -12,8 +12,9 @@
     <sheet name="ChiPhi" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="PERT" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Gantt" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="RuiRo" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="MaTran" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="NenLich" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="RuiRo" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="MaTran" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -87,7 +88,7 @@
       <sz val="7"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -112,6 +113,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00EEF3FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
@@ -214,7 +220,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -296,6 +302,10 @@
     </xf>
     <xf numFmtId="169" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="170" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -311,13 +321,13 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -751,7 +761,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:C20"/>
+  <dimension ref="B2:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -880,54 +890,66 @@
     <row r="15">
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>RuiRo</t>
+          <t>NenLich</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Sổ đăng ký rủi ro (Risk Register), sắp theo điểm giảm dần. 2 dòng cuối để nhóm tự bổ sung.</t>
+          <t>Kịch bản nén lịch (fast-tracking + giảm phạm vi) – lịch mới, đường găng mới, xác suất kịp hạn.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="3" t="inlineStr">
         <is>
+          <t>RuiRo</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Sổ đăng ký rủi ro (Risk Register), sắp theo điểm giảm dần. 2 dòng cuối để nhóm tự bổ sung.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="3" t="inlineStr">
+        <is>
           <t>MaTran</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>Ma trận xác suất × tác động 5×5, tự điền mã rủi ro theo sheet RuiRo.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="B17" s="3" t="inlineStr"/>
-      <c r="C17" s="4" t="inlineStr"/>
-    </row>
     <row r="18">
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr"/>
+      <c r="C18" s="4" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>Lưu ý</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>Các số O/M/P, giờ công, đơn giá là GIẢ ĐỊNH do AI đề xuất làm bản nháp – nhóm cần xem lại và điều chỉnh theo ý kiến của nhóm.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" s="3" t="inlineStr"/>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>Nếu sửa XS/TĐ trong sheet RuiRo, hãy sắp xếp lại bảng theo cột Điểm (Data → Sort) để đúng yêu cầu "sắp theo điểm giảm dần".</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="3" t="inlineStr"/>
       <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Nếu sửa XS/TĐ trong sheet RuiRo, hãy sắp xếp lại bảng theo cột Điểm (Data → Sort) để đúng yêu cầu "sắp theo điểm giảm dần".</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="3" t="inlineStr"/>
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>Nếu thêm/bớt hoạt động PERT, phải sửa lại công thức ES (MAX EF của hoạt động trước) và LF (MIN LS của hoạt động sau).</t>
         </is>
@@ -11488,6 +11510,1243 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:P29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="6" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+    <col width="8" customWidth="1" min="13" max="13"/>
+    <col width="8" customWidth="1" min="14" max="14"/>
+    <col width="8" customWidth="1" min="15" max="15"/>
+    <col width="70" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PHƯƠNG ÁN NÉN LỊCH – fast-tracking + giảm phạm vi (AI đề xuất, nhóm xác nhận)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Cột "Chồng lấn" = số ngày hoạt động được bắt đầu SỚM trước khi các hoạt động trước kết thúc (fast-tracking). ES = MAX(0; MAX(EF hoạt động trước) − Chồng lấn); LF = MIN(LS hoạt động sau + Chồng lấn của hoạt động sau). Sheet PERT giữ nguyên làm lịch gốc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Mã</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Hoạt động</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Trước</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>Chồng lấn</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>TE</t>
+        </is>
+      </c>
+      <c r="I4" s="7" t="inlineStr">
+        <is>
+          <t>σ²</t>
+        </is>
+      </c>
+      <c r="J4" s="7" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="K4" s="7" t="inlineStr">
+        <is>
+          <t>EF</t>
+        </is>
+      </c>
+      <c r="L4" s="7" t="inlineStr">
+        <is>
+          <t>LS</t>
+        </is>
+      </c>
+      <c r="M4" s="7" t="inlineStr">
+        <is>
+          <t>LF</t>
+        </is>
+      </c>
+      <c r="N4" s="7" t="inlineStr">
+        <is>
+          <t>Slack</t>
+        </is>
+      </c>
+      <c r="O4" s="7" t="inlineStr">
+        <is>
+          <t>Găng?</t>
+        </is>
+      </c>
+      <c r="P4" s="7" t="inlineStr">
+        <is>
+          <t>Thay đổi so với lịch gốc</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="28" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B5" s="24">
+        <f>PERT!B9</f>
+        <v/>
+      </c>
+      <c r="C5" s="23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D5" s="51">
+        <f>PERT!E9</f>
+        <v/>
+      </c>
+      <c r="E5" s="51">
+        <f>PERT!F9</f>
+        <v/>
+      </c>
+      <c r="F5" s="51">
+        <f>PERT!G9</f>
+        <v/>
+      </c>
+      <c r="G5" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="38">
+        <f>(D5+4*E5+F5)/6</f>
+        <v/>
+      </c>
+      <c r="I5" s="38">
+        <f>((F5-D5)/6)^2</f>
+        <v/>
+      </c>
+      <c r="J5" s="38">
+        <f>0</f>
+        <v/>
+      </c>
+      <c r="K5" s="38">
+        <f>J5+H5</f>
+        <v/>
+      </c>
+      <c r="L5" s="38">
+        <f>M5-H5</f>
+        <v/>
+      </c>
+      <c r="M5" s="38">
+        <f>MIN(L6+G6)</f>
+        <v/>
+      </c>
+      <c r="N5" s="38">
+        <f>L5-J5</f>
+        <v/>
+      </c>
+      <c r="O5" s="28">
+        <f>IF(ABS(N5)&lt;0.005,"Găng","")</f>
+        <v/>
+      </c>
+      <c r="P5" s="24" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="28" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B6" s="24">
+        <f>PERT!B10</f>
+        <v/>
+      </c>
+      <c r="C6" s="23" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D6" s="51">
+        <f>PERT!E10</f>
+        <v/>
+      </c>
+      <c r="E6" s="51">
+        <f>PERT!F10</f>
+        <v/>
+      </c>
+      <c r="F6" s="51">
+        <f>PERT!G10</f>
+        <v/>
+      </c>
+      <c r="G6" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="38">
+        <f>(D6+4*E6+F6)/6</f>
+        <v/>
+      </c>
+      <c r="I6" s="38">
+        <f>((F6-D6)/6)^2</f>
+        <v/>
+      </c>
+      <c r="J6" s="38">
+        <f>MAX(0,MAX(K5)-G6)</f>
+        <v/>
+      </c>
+      <c r="K6" s="38">
+        <f>J6+H6</f>
+        <v/>
+      </c>
+      <c r="L6" s="38">
+        <f>M6-H6</f>
+        <v/>
+      </c>
+      <c r="M6" s="38">
+        <f>MIN(L7+G7)</f>
+        <v/>
+      </c>
+      <c r="N6" s="38">
+        <f>L6-J6</f>
+        <v/>
+      </c>
+      <c r="O6" s="28">
+        <f>IF(ABS(N6)&lt;0.005,"Găng","")</f>
+        <v/>
+      </c>
+      <c r="P6" s="24" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="28" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B7" s="24">
+        <f>PERT!B11</f>
+        <v/>
+      </c>
+      <c r="C7" s="23" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D7" s="51">
+        <f>PERT!E11</f>
+        <v/>
+      </c>
+      <c r="E7" s="51">
+        <f>PERT!F11</f>
+        <v/>
+      </c>
+      <c r="F7" s="51">
+        <f>PERT!G11</f>
+        <v/>
+      </c>
+      <c r="G7" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="38">
+        <f>(D7+4*E7+F7)/6</f>
+        <v/>
+      </c>
+      <c r="I7" s="38">
+        <f>((F7-D7)/6)^2</f>
+        <v/>
+      </c>
+      <c r="J7" s="38">
+        <f>MAX(0,MAX(K6)-G7)</f>
+        <v/>
+      </c>
+      <c r="K7" s="38">
+        <f>J7+H7</f>
+        <v/>
+      </c>
+      <c r="L7" s="38">
+        <f>M7-H7</f>
+        <v/>
+      </c>
+      <c r="M7" s="38">
+        <f>MIN(L8+G8,L9+G9,L16+G16)</f>
+        <v/>
+      </c>
+      <c r="N7" s="38">
+        <f>L7-J7</f>
+        <v/>
+      </c>
+      <c r="O7" s="28">
+        <f>IF(ABS(N7)&lt;0.005,"Găng","")</f>
+        <v/>
+      </c>
+      <c r="P7" s="24" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="28" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B8" s="24">
+        <f>PERT!B12</f>
+        <v/>
+      </c>
+      <c r="C8" s="23" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D8" s="51">
+        <f>PERT!E12</f>
+        <v/>
+      </c>
+      <c r="E8" s="51">
+        <f>PERT!F12</f>
+        <v/>
+      </c>
+      <c r="F8" s="51">
+        <f>PERT!G12</f>
+        <v/>
+      </c>
+      <c r="G8" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="H8" s="38">
+        <f>(D8+4*E8+F8)/6</f>
+        <v/>
+      </c>
+      <c r="I8" s="38">
+        <f>((F8-D8)/6)^2</f>
+        <v/>
+      </c>
+      <c r="J8" s="38">
+        <f>MAX(0,MAX(K7)-G8)</f>
+        <v/>
+      </c>
+      <c r="K8" s="38">
+        <f>J8+H8</f>
+        <v/>
+      </c>
+      <c r="L8" s="38">
+        <f>M8-H8</f>
+        <v/>
+      </c>
+      <c r="M8" s="38">
+        <f>MIN(L10+G10)</f>
+        <v/>
+      </c>
+      <c r="N8" s="38">
+        <f>L8-J8</f>
+        <v/>
+      </c>
+      <c r="O8" s="28">
+        <f>IF(ABS(N8)&lt;0.005,"Găng","")</f>
+        <v/>
+      </c>
+      <c r="P8" s="24" t="inlineStr">
+        <is>
+          <t>Fast-tracking: thiết kế kiến trúc bắt đầu khi SRS đã duyệt phần lõi (FR01–FR08)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="28" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="B9" s="24">
+        <f>PERT!B13</f>
+        <v/>
+      </c>
+      <c r="C9" s="23" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D9" s="51">
+        <f>PERT!E13</f>
+        <v/>
+      </c>
+      <c r="E9" s="51">
+        <f>PERT!F13</f>
+        <v/>
+      </c>
+      <c r="F9" s="51">
+        <f>PERT!G13</f>
+        <v/>
+      </c>
+      <c r="G9" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="H9" s="38">
+        <f>(D9+4*E9+F9)/6</f>
+        <v/>
+      </c>
+      <c r="I9" s="38">
+        <f>((F9-D9)/6)^2</f>
+        <v/>
+      </c>
+      <c r="J9" s="38">
+        <f>MAX(0,MAX(K7)-G9)</f>
+        <v/>
+      </c>
+      <c r="K9" s="38">
+        <f>J9+H9</f>
+        <v/>
+      </c>
+      <c r="L9" s="38">
+        <f>M9-H9</f>
+        <v/>
+      </c>
+      <c r="M9" s="38">
+        <f>MIN(L13+G13)</f>
+        <v/>
+      </c>
+      <c r="N9" s="38">
+        <f>L9-J9</f>
+        <v/>
+      </c>
+      <c r="O9" s="28">
+        <f>IF(ABS(N9)&lt;0.005,"Găng","")</f>
+        <v/>
+      </c>
+      <c r="P9" s="24" t="inlineStr">
+        <is>
+          <t>Fast-tracking: thiết kế giao diện bắt đầu song song giai đoạn cuối SRS</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="28" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="B10" s="24">
+        <f>PERT!B14</f>
+        <v/>
+      </c>
+      <c r="C10" s="23" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="D10" s="51">
+        <f>PERT!E14</f>
+        <v/>
+      </c>
+      <c r="E10" s="51">
+        <f>PERT!F14</f>
+        <v/>
+      </c>
+      <c r="F10" s="51">
+        <f>PERT!G14</f>
+        <v/>
+      </c>
+      <c r="G10" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="38">
+        <f>(D10+4*E10+F10)/6</f>
+        <v/>
+      </c>
+      <c r="I10" s="38">
+        <f>((F10-D10)/6)^2</f>
+        <v/>
+      </c>
+      <c r="J10" s="38">
+        <f>MAX(0,MAX(K8)-G10)</f>
+        <v/>
+      </c>
+      <c r="K10" s="38">
+        <f>J10+H10</f>
+        <v/>
+      </c>
+      <c r="L10" s="38">
+        <f>M10-H10</f>
+        <v/>
+      </c>
+      <c r="M10" s="38">
+        <f>MIN(L11+G11,L12+G12,L14+G14)</f>
+        <v/>
+      </c>
+      <c r="N10" s="38">
+        <f>L10-J10</f>
+        <v/>
+      </c>
+      <c r="O10" s="28">
+        <f>IF(ABS(N10)&lt;0.005,"Găng","")</f>
+        <v/>
+      </c>
+      <c r="P10" s="24" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="28" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="B11" s="24">
+        <f>PERT!B15</f>
+        <v/>
+      </c>
+      <c r="C11" s="23" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D11" s="54" t="n">
+        <v>12</v>
+      </c>
+      <c r="E11" s="54" t="n">
+        <v>15</v>
+      </c>
+      <c r="F11" s="54" t="n">
+        <v>22</v>
+      </c>
+      <c r="G11" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="38">
+        <f>(D11+4*E11+F11)/6</f>
+        <v/>
+      </c>
+      <c r="I11" s="38">
+        <f>((F11-D11)/6)^2</f>
+        <v/>
+      </c>
+      <c r="J11" s="38">
+        <f>MAX(0,MAX(K10)-G11)</f>
+        <v/>
+      </c>
+      <c r="K11" s="38">
+        <f>J11+H11</f>
+        <v/>
+      </c>
+      <c r="L11" s="38">
+        <f>M11-H11</f>
+        <v/>
+      </c>
+      <c r="M11" s="38">
+        <f>MIN(L15+G15)</f>
+        <v/>
+      </c>
+      <c r="N11" s="38">
+        <f>L11-J11</f>
+        <v/>
+      </c>
+      <c r="O11" s="28">
+        <f>IF(ABS(N11)&lt;0.005,"Găng","")</f>
+        <v/>
+      </c>
+      <c r="P11" s="24" t="inlineStr">
+        <is>
+          <t>Giảm phạm vi: dời API khách hàng thân thiết, nhân viên/ca (FR09–FR10) sang giai đoạn 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="28" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="B12" s="24">
+        <f>PERT!B16</f>
+        <v/>
+      </c>
+      <c r="C12" s="23" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D12" s="51">
+        <f>PERT!E16</f>
+        <v/>
+      </c>
+      <c r="E12" s="51">
+        <f>PERT!F16</f>
+        <v/>
+      </c>
+      <c r="F12" s="51">
+        <f>PERT!G16</f>
+        <v/>
+      </c>
+      <c r="G12" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="38">
+        <f>(D12+4*E12+F12)/6</f>
+        <v/>
+      </c>
+      <c r="I12" s="38">
+        <f>((F12-D12)/6)^2</f>
+        <v/>
+      </c>
+      <c r="J12" s="38">
+        <f>MAX(0,MAX(K10)-G12)</f>
+        <v/>
+      </c>
+      <c r="K12" s="38">
+        <f>J12+H12</f>
+        <v/>
+      </c>
+      <c r="L12" s="38">
+        <f>M12-H12</f>
+        <v/>
+      </c>
+      <c r="M12" s="38">
+        <f>MIN(L17+G17)</f>
+        <v/>
+      </c>
+      <c r="N12" s="38">
+        <f>L12-J12</f>
+        <v/>
+      </c>
+      <c r="O12" s="28">
+        <f>IF(ABS(N12)&lt;0.005,"Găng","")</f>
+        <v/>
+      </c>
+      <c r="P12" s="24" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="28" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="B13" s="24">
+        <f>PERT!B17</f>
+        <v/>
+      </c>
+      <c r="C13" s="23" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="D13" s="51">
+        <f>PERT!E17</f>
+        <v/>
+      </c>
+      <c r="E13" s="51">
+        <f>PERT!F17</f>
+        <v/>
+      </c>
+      <c r="F13" s="51">
+        <f>PERT!G17</f>
+        <v/>
+      </c>
+      <c r="G13" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="38">
+        <f>(D13+4*E13+F13)/6</f>
+        <v/>
+      </c>
+      <c r="I13" s="38">
+        <f>((F13-D13)/6)^2</f>
+        <v/>
+      </c>
+      <c r="J13" s="38">
+        <f>MAX(0,MAX(K9)-G13)</f>
+        <v/>
+      </c>
+      <c r="K13" s="38">
+        <f>J13+H13</f>
+        <v/>
+      </c>
+      <c r="L13" s="38">
+        <f>M13-H13</f>
+        <v/>
+      </c>
+      <c r="M13" s="38">
+        <f>MIN(L14+G14)</f>
+        <v/>
+      </c>
+      <c r="N13" s="38">
+        <f>L13-J13</f>
+        <v/>
+      </c>
+      <c r="O13" s="28">
+        <f>IF(ABS(N13)&lt;0.005,"Găng","")</f>
+        <v/>
+      </c>
+      <c r="P13" s="24" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="28" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="B14" s="24">
+        <f>PERT!B18</f>
+        <v/>
+      </c>
+      <c r="C14" s="23" t="inlineStr">
+        <is>
+          <t>I, F</t>
+        </is>
+      </c>
+      <c r="D14" s="54" t="n">
+        <v>12</v>
+      </c>
+      <c r="E14" s="54" t="n">
+        <v>16</v>
+      </c>
+      <c r="F14" s="54" t="n">
+        <v>23</v>
+      </c>
+      <c r="G14" s="53" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="H14" s="38">
+        <f>(D14+4*E14+F14)/6</f>
+        <v/>
+      </c>
+      <c r="I14" s="38">
+        <f>((F14-D14)/6)^2</f>
+        <v/>
+      </c>
+      <c r="J14" s="38">
+        <f>MAX(0,MAX(K13,K10)-G14)</f>
+        <v/>
+      </c>
+      <c r="K14" s="38">
+        <f>J14+H14</f>
+        <v/>
+      </c>
+      <c r="L14" s="38">
+        <f>M14-H14</f>
+        <v/>
+      </c>
+      <c r="M14" s="38">
+        <f>MIN(L17+G17)</f>
+        <v/>
+      </c>
+      <c r="N14" s="38">
+        <f>L14-J14</f>
+        <v/>
+      </c>
+      <c r="O14" s="28">
+        <f>IF(ABS(N14)&lt;0.005,"Găng","")</f>
+        <v/>
+      </c>
+      <c r="P14" s="24" t="inlineStr">
+        <is>
+          <t>Giảm phạm vi FR09–FR10 + fast-tracking: làm màn hình trên mockup và API giả lập khi khung giao diện xong khoảng 50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="28" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="B15" s="24">
+        <f>PERT!B19</f>
+        <v/>
+      </c>
+      <c r="C15" s="23" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="D15" s="51">
+        <f>PERT!E19</f>
+        <v/>
+      </c>
+      <c r="E15" s="51">
+        <f>PERT!F19</f>
+        <v/>
+      </c>
+      <c r="F15" s="51">
+        <f>PERT!G19</f>
+        <v/>
+      </c>
+      <c r="G15" s="53" t="n">
+        <v>3</v>
+      </c>
+      <c r="H15" s="38">
+        <f>(D15+4*E15+F15)/6</f>
+        <v/>
+      </c>
+      <c r="I15" s="38">
+        <f>((F15-D15)/6)^2</f>
+        <v/>
+      </c>
+      <c r="J15" s="38">
+        <f>MAX(0,MAX(K11)-G15)</f>
+        <v/>
+      </c>
+      <c r="K15" s="38">
+        <f>J15+H15</f>
+        <v/>
+      </c>
+      <c r="L15" s="38">
+        <f>M15-H15</f>
+        <v/>
+      </c>
+      <c r="M15" s="38">
+        <f>MIN(L17+G17)</f>
+        <v/>
+      </c>
+      <c r="N15" s="38">
+        <f>L15-J15</f>
+        <v/>
+      </c>
+      <c r="O15" s="28">
+        <f>IF(ABS(N15)&lt;0.005,"Găng","")</f>
+        <v/>
+      </c>
+      <c r="P15" s="24" t="inlineStr">
+        <is>
+          <t>Fast-tracking: xuất báo cáo làm khi API doanh thu, tồn kho đã xong (không chờ toàn bộ API)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="28" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="B16" s="24">
+        <f>PERT!B20</f>
+        <v/>
+      </c>
+      <c r="C16" s="23" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D16" s="51">
+        <f>PERT!E20</f>
+        <v/>
+      </c>
+      <c r="E16" s="51">
+        <f>PERT!F20</f>
+        <v/>
+      </c>
+      <c r="F16" s="51">
+        <f>PERT!G20</f>
+        <v/>
+      </c>
+      <c r="G16" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="38">
+        <f>(D16+4*E16+F16)/6</f>
+        <v/>
+      </c>
+      <c r="I16" s="38">
+        <f>((F16-D16)/6)^2</f>
+        <v/>
+      </c>
+      <c r="J16" s="38">
+        <f>MAX(0,MAX(K7)-G16)</f>
+        <v/>
+      </c>
+      <c r="K16" s="38">
+        <f>J16+H16</f>
+        <v/>
+      </c>
+      <c r="L16" s="38">
+        <f>M16-H16</f>
+        <v/>
+      </c>
+      <c r="M16" s="38">
+        <f>MIN(L17+G17)</f>
+        <v/>
+      </c>
+      <c r="N16" s="38">
+        <f>L16-J16</f>
+        <v/>
+      </c>
+      <c r="O16" s="28">
+        <f>IF(ABS(N16)&lt;0.005,"Găng","")</f>
+        <v/>
+      </c>
+      <c r="P16" s="24" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="28" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="B17" s="24">
+        <f>PERT!B21</f>
+        <v/>
+      </c>
+      <c r="C17" s="23" t="inlineStr">
+        <is>
+          <t>J, K, H, L</t>
+        </is>
+      </c>
+      <c r="D17" s="51">
+        <f>PERT!E21</f>
+        <v/>
+      </c>
+      <c r="E17" s="51">
+        <f>PERT!F21</f>
+        <v/>
+      </c>
+      <c r="F17" s="51">
+        <f>PERT!G21</f>
+        <v/>
+      </c>
+      <c r="G17" s="53" t="n">
+        <v>5</v>
+      </c>
+      <c r="H17" s="38">
+        <f>(D17+4*E17+F17)/6</f>
+        <v/>
+      </c>
+      <c r="I17" s="38">
+        <f>((F17-D17)/6)^2</f>
+        <v/>
+      </c>
+      <c r="J17" s="38">
+        <f>MAX(0,MAX(K14,K15,K12,K16)-G17)</f>
+        <v/>
+      </c>
+      <c r="K17" s="38">
+        <f>J17+H17</f>
+        <v/>
+      </c>
+      <c r="L17" s="38">
+        <f>M17-H17</f>
+        <v/>
+      </c>
+      <c r="M17" s="38">
+        <f>MIN(L18+G18)</f>
+        <v/>
+      </c>
+      <c r="N17" s="38">
+        <f>L17-J17</f>
+        <v/>
+      </c>
+      <c r="O17" s="28">
+        <f>IF(ABS(N17)&lt;0.005,"Găng","")</f>
+        <v/>
+      </c>
+      <c r="P17" s="24" t="inlineStr">
+        <is>
+          <t>Fast-tracking: kiểm thử theo từng module xong trước, chồng 5 ngày cuối giai đoạn phát triển</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="28" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="B18" s="24">
+        <f>PERT!B22</f>
+        <v/>
+      </c>
+      <c r="C18" s="23" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D18" s="51">
+        <f>PERT!E22</f>
+        <v/>
+      </c>
+      <c r="E18" s="51">
+        <f>PERT!F22</f>
+        <v/>
+      </c>
+      <c r="F18" s="51">
+        <f>PERT!G22</f>
+        <v/>
+      </c>
+      <c r="G18" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="38">
+        <f>(D18+4*E18+F18)/6</f>
+        <v/>
+      </c>
+      <c r="I18" s="38">
+        <f>((F18-D18)/6)^2</f>
+        <v/>
+      </c>
+      <c r="J18" s="38">
+        <f>MAX(0,MAX(K17)-G18)</f>
+        <v/>
+      </c>
+      <c r="K18" s="38">
+        <f>J18+H18</f>
+        <v/>
+      </c>
+      <c r="L18" s="38">
+        <f>M18-H18</f>
+        <v/>
+      </c>
+      <c r="M18" s="38">
+        <f>MIN(L19+G19)</f>
+        <v/>
+      </c>
+      <c r="N18" s="38">
+        <f>L18-J18</f>
+        <v/>
+      </c>
+      <c r="O18" s="28">
+        <f>IF(ABS(N18)&lt;0.005,"Găng","")</f>
+        <v/>
+      </c>
+      <c r="P18" s="24" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="28" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="B19" s="24">
+        <f>PERT!B23</f>
+        <v/>
+      </c>
+      <c r="C19" s="23" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="D19" s="51">
+        <f>PERT!E23</f>
+        <v/>
+      </c>
+      <c r="E19" s="51">
+        <f>PERT!F23</f>
+        <v/>
+      </c>
+      <c r="F19" s="51">
+        <f>PERT!G23</f>
+        <v/>
+      </c>
+      <c r="G19" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="38">
+        <f>(D19+4*E19+F19)/6</f>
+        <v/>
+      </c>
+      <c r="I19" s="38">
+        <f>((F19-D19)/6)^2</f>
+        <v/>
+      </c>
+      <c r="J19" s="38">
+        <f>MAX(0,MAX(K18)-G19)</f>
+        <v/>
+      </c>
+      <c r="K19" s="38">
+        <f>J19+H19</f>
+        <v/>
+      </c>
+      <c r="L19" s="38">
+        <f>M19-H19</f>
+        <v/>
+      </c>
+      <c r="M19" s="38">
+        <f>$C$22</f>
+        <v/>
+      </c>
+      <c r="N19" s="38">
+        <f>L19-J19</f>
+        <v/>
+      </c>
+      <c r="O19" s="28">
+        <f>IF(ABS(N19)&lt;0.005,"Găng","")</f>
+        <v/>
+      </c>
+      <c r="P19" s="24" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>KẾT QUẢ SAU KHI NÉN</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="26" t="inlineStr">
+        <is>
+          <t>Thời gian dự án T mới (ngày làm việc)</t>
+        </is>
+      </c>
+      <c r="B22" s="41" t="n"/>
+      <c r="C22" s="42">
+        <f>MAX(K5:K19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="26" t="inlineStr">
+        <is>
+          <t>Đường găng mới</t>
+        </is>
+      </c>
+      <c r="B23" s="41" t="n"/>
+      <c r="C23" s="26">
+        <f>LEFT(IF(O5="Găng","A → ","")&amp;IF(O6="Găng","B → ","")&amp;IF(O7="Găng","C → ","")&amp;IF(O8="Găng","D → ","")&amp;IF(O9="Găng","E → ","")&amp;IF(O10="Găng","F → ","")&amp;IF(O11="Găng","G → ","")&amp;IF(O12="Găng","H → ","")&amp;IF(O13="Găng","I → ","")&amp;IF(O14="Găng","J → ","")&amp;IF(O15="Găng","K → ","")&amp;IF(O16="Găng","L → ","")&amp;IF(O17="Găng","M → ","")&amp;IF(O18="Găng","N → ","")&amp;IF(O19="Găng","O → ",""),LEN(IF(O5="Găng","A → ","")&amp;IF(O6="Găng","B → ","")&amp;IF(O7="Găng","C → ","")&amp;IF(O8="Găng","D → ","")&amp;IF(O9="Găng","E → ","")&amp;IF(O10="Găng","F → ","")&amp;IF(O11="Găng","G → ","")&amp;IF(O12="Găng","H → ","")&amp;IF(O13="Găng","I → ","")&amp;IF(O14="Găng","J → ","")&amp;IF(O15="Găng","K → ","")&amp;IF(O16="Găng","L → ","")&amp;IF(O17="Găng","M → ","")&amp;IF(O18="Găng","N → ","")&amp;IF(O19="Găng","O → ",""))-3)</f>
+        <v/>
+      </c>
+      <c r="D23" s="43" t="n"/>
+      <c r="E23" s="43" t="n"/>
+      <c r="F23" s="43" t="n"/>
+      <c r="G23" s="43" t="n"/>
+      <c r="H23" s="43" t="n"/>
+      <c r="I23" s="43" t="n"/>
+      <c r="J23" s="44" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="26" t="inlineStr">
+        <is>
+          <t>Độ lệch chuẩn đường găng σ</t>
+        </is>
+      </c>
+      <c r="B24" s="41" t="n"/>
+      <c r="C24" s="42">
+        <f>SQRT(SUMIF(O5:O19,"Găng",I5:I19))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="26" t="inlineStr">
+        <is>
+          <t>Số ngày làm việc tới hạn chót</t>
+        </is>
+      </c>
+      <c r="B25" s="41" t="n"/>
+      <c r="C25" s="29">
+        <f>PERT!C5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="26" t="inlineStr">
+        <is>
+          <t>Dự trữ so với hạn chót (ngày)</t>
+        </is>
+      </c>
+      <c r="B26" s="41" t="n"/>
+      <c r="C26" s="42">
+        <f>C25-C22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="26" t="inlineStr">
+        <is>
+          <t>Xác suất kịp hạn P(Z)</t>
+        </is>
+      </c>
+      <c r="B27" s="41" t="n"/>
+      <c r="C27" s="35">
+        <f>NORMSDIST((C25-C22)/C24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="26" t="inlineStr">
+        <is>
+          <t>Ngày kết thúc dự kiến</t>
+        </is>
+      </c>
+      <c r="B28" s="41" t="n"/>
+      <c r="C28" s="46">
+        <f>WORKDAY(PERT!C3,ROUNDUP(C22,0)-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="26" t="inlineStr">
+        <is>
+          <t>T lịch gốc (sheet PERT) / số ngày rút ngắn</t>
+        </is>
+      </c>
+      <c r="B29" s="41" t="n"/>
+      <c r="C29" s="42">
+        <f>PERT!$C$26</f>
+        <v/>
+      </c>
+      <c r="D29" s="42">
+        <f>C29-C22</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="C23:J23"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A2:P2"/>
+  </mergeCells>
+  <conditionalFormatting sqref="A5:O19">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>$O5="Găng"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:M16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -11588,7 +12847,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="51" t="inlineStr">
+      <c r="A5" s="55" t="inlineStr">
         <is>
           <t>R01</t>
         </is>
@@ -11613,13 +12872,13 @@
           <t>Bên ngoài / Kỹ thuật</t>
         </is>
       </c>
-      <c r="F5" s="52" t="n">
+      <c r="F5" s="56" t="n">
         <v>4</v>
       </c>
-      <c r="G5" s="52" t="n">
+      <c r="G5" s="56" t="n">
         <v>5</v>
       </c>
-      <c r="H5" s="53">
+      <c r="H5" s="57">
         <f>F5*G5</f>
         <v/>
       </c>
@@ -11649,7 +12908,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="51" t="inlineStr">
+      <c r="A6" s="55" t="inlineStr">
         <is>
           <t>R02</t>
         </is>
@@ -11674,13 +12933,13 @@
           <t>Lịch trình</t>
         </is>
       </c>
-      <c r="F6" s="52" t="n">
+      <c r="F6" s="56" t="n">
         <v>4</v>
       </c>
-      <c r="G6" s="52" t="n">
+      <c r="G6" s="56" t="n">
         <v>4</v>
       </c>
-      <c r="H6" s="53">
+      <c r="H6" s="57">
         <f>F6*G6</f>
         <v/>
       </c>
@@ -11710,7 +12969,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="51" t="inlineStr">
+      <c r="A7" s="55" t="inlineStr">
         <is>
           <t>R03</t>
         </is>
@@ -11735,13 +12994,13 @@
           <t>Khách hàng / Yêu cầu</t>
         </is>
       </c>
-      <c r="F7" s="52" t="n">
+      <c r="F7" s="56" t="n">
         <v>4</v>
       </c>
-      <c r="G7" s="52" t="n">
+      <c r="G7" s="56" t="n">
         <v>4</v>
       </c>
-      <c r="H7" s="53">
+      <c r="H7" s="57">
         <f>F7*G7</f>
         <v/>
       </c>
@@ -11771,7 +13030,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="51" t="inlineStr">
+      <c r="A8" s="55" t="inlineStr">
         <is>
           <t>R04</t>
         </is>
@@ -11796,13 +13055,13 @@
           <t>Kỹ thuật / Dữ liệu</t>
         </is>
       </c>
-      <c r="F8" s="52" t="n">
+      <c r="F8" s="56" t="n">
         <v>4</v>
       </c>
-      <c r="G8" s="52" t="n">
+      <c r="G8" s="56" t="n">
         <v>4</v>
       </c>
-      <c r="H8" s="53">
+      <c r="H8" s="57">
         <f>F8*G8</f>
         <v/>
       </c>
@@ -11832,7 +13091,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="51" t="inlineStr">
+      <c r="A9" s="55" t="inlineStr">
         <is>
           <t>R05</t>
         </is>
@@ -11857,13 +13116,13 @@
           <t>Con người</t>
         </is>
       </c>
-      <c r="F9" s="52" t="n">
+      <c r="F9" s="56" t="n">
         <v>3</v>
       </c>
-      <c r="G9" s="52" t="n">
+      <c r="G9" s="56" t="n">
         <v>5</v>
       </c>
-      <c r="H9" s="53">
+      <c r="H9" s="57">
         <f>F9*G9</f>
         <v/>
       </c>
@@ -11893,7 +13152,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="51" t="inlineStr">
+      <c r="A10" s="55" t="inlineStr">
         <is>
           <t>R06</t>
         </is>
@@ -11918,13 +13177,13 @@
           <t>Bảo mật / Pháp lý</t>
         </is>
       </c>
-      <c r="F10" s="52" t="n">
+      <c r="F10" s="56" t="n">
         <v>2</v>
       </c>
-      <c r="G10" s="52" t="n">
+      <c r="G10" s="56" t="n">
         <v>5</v>
       </c>
-      <c r="H10" s="53">
+      <c r="H10" s="57">
         <f>F10*G10</f>
         <v/>
       </c>
@@ -11954,7 +13213,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="51" t="inlineStr">
+      <c r="A11" s="55" t="inlineStr">
         <is>
           <t>R07</t>
         </is>
@@ -11979,13 +13238,13 @@
           <t>Con người / Khách hàng</t>
         </is>
       </c>
-      <c r="F11" s="52" t="n">
+      <c r="F11" s="56" t="n">
         <v>3</v>
       </c>
-      <c r="G11" s="52" t="n">
+      <c r="G11" s="56" t="n">
         <v>3</v>
       </c>
-      <c r="H11" s="53">
+      <c r="H11" s="57">
         <f>F11*G11</f>
         <v/>
       </c>
@@ -12015,7 +13274,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="51" t="inlineStr">
+      <c r="A12" s="55" t="inlineStr">
         <is>
           <t>R08</t>
         </is>
@@ -12040,13 +13299,13 @@
           <t>Kỹ thuật</t>
         </is>
       </c>
-      <c r="F12" s="52" t="n">
+      <c r="F12" s="56" t="n">
         <v>3</v>
       </c>
-      <c r="G12" s="52" t="n">
+      <c r="G12" s="56" t="n">
         <v>3</v>
       </c>
-      <c r="H12" s="53">
+      <c r="H12" s="57">
         <f>F12*G12</f>
         <v/>
       </c>
@@ -12076,7 +13335,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="51" t="inlineStr">
+      <c r="A13" s="55" t="inlineStr">
         <is>
           <t>R09</t>
         </is>
@@ -12101,13 +13360,13 @@
           <t>Khách hàng / Pháp lý</t>
         </is>
       </c>
-      <c r="F13" s="52" t="n">
+      <c r="F13" s="56" t="n">
         <v>2</v>
       </c>
-      <c r="G13" s="52" t="n">
+      <c r="G13" s="56" t="n">
         <v>4</v>
       </c>
-      <c r="H13" s="53">
+      <c r="H13" s="57">
         <f>F13*G13</f>
         <v/>
       </c>
@@ -12137,7 +13396,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="51" t="inlineStr">
+      <c r="A14" s="55" t="inlineStr">
         <is>
           <t>R10</t>
         </is>
@@ -12162,13 +13421,13 @@
           <t>Bên ngoài / Hạ tầng</t>
         </is>
       </c>
-      <c r="F14" s="52" t="n">
+      <c r="F14" s="56" t="n">
         <v>2</v>
       </c>
-      <c r="G14" s="52" t="n">
+      <c r="G14" s="56" t="n">
         <v>3</v>
       </c>
-      <c r="H14" s="53">
+      <c r="H14" s="57">
         <f>F14*G14</f>
         <v/>
       </c>
@@ -12203,24 +13462,24 @@
           <t>R11</t>
         </is>
       </c>
-      <c r="B15" s="54" t="n"/>
-      <c r="C15" s="54" t="n"/>
-      <c r="D15" s="54" t="n"/>
-      <c r="E15" s="54" t="n"/>
-      <c r="F15" s="54" t="n"/>
-      <c r="G15" s="54" t="n"/>
-      <c r="H15" s="54">
+      <c r="B15" s="58" t="n"/>
+      <c r="C15" s="58" t="n"/>
+      <c r="D15" s="58" t="n"/>
+      <c r="E15" s="58" t="n"/>
+      <c r="F15" s="58" t="n"/>
+      <c r="G15" s="58" t="n"/>
+      <c r="H15" s="58">
         <f>IF(OR(F15="",G15=""),"",F15*G15)</f>
         <v/>
       </c>
-      <c r="I15" s="54">
+      <c r="I15" s="58">
         <f>IF(H15="","",IF(H15&gt;=15,"Cao",IF(H15&gt;=8,"Trung bình","Thấp")))</f>
         <v/>
       </c>
-      <c r="J15" s="54" t="n"/>
-      <c r="K15" s="54" t="n"/>
-      <c r="L15" s="54" t="n"/>
-      <c r="M15" s="54" t="inlineStr">
+      <c r="J15" s="58" t="n"/>
+      <c r="K15" s="58" t="n"/>
+      <c r="L15" s="58" t="n"/>
+      <c r="M15" s="58" t="inlineStr">
         <is>
           <t>Nhóm bổ sung</t>
         </is>
@@ -12232,24 +13491,24 @@
           <t>R12</t>
         </is>
       </c>
-      <c r="B16" s="54" t="n"/>
-      <c r="C16" s="54" t="n"/>
-      <c r="D16" s="54" t="n"/>
-      <c r="E16" s="54" t="n"/>
-      <c r="F16" s="54" t="n"/>
-      <c r="G16" s="54" t="n"/>
-      <c r="H16" s="54">
+      <c r="B16" s="58" t="n"/>
+      <c r="C16" s="58" t="n"/>
+      <c r="D16" s="58" t="n"/>
+      <c r="E16" s="58" t="n"/>
+      <c r="F16" s="58" t="n"/>
+      <c r="G16" s="58" t="n"/>
+      <c r="H16" s="58">
         <f>IF(OR(F16="",G16=""),"",F16*G16)</f>
         <v/>
       </c>
-      <c r="I16" s="54">
+      <c r="I16" s="58">
         <f>IF(H16="","",IF(H16&gt;=15,"Cao",IF(H16&gt;=8,"Trung bình","Thấp")))</f>
         <v/>
       </c>
-      <c r="J16" s="54" t="n"/>
-      <c r="K16" s="54" t="n"/>
-      <c r="L16" s="54" t="n"/>
-      <c r="M16" s="54" t="inlineStr">
+      <c r="J16" s="58" t="n"/>
+      <c r="K16" s="58" t="n"/>
+      <c r="L16" s="58" t="n"/>
+      <c r="M16" s="58" t="inlineStr">
         <is>
           <t>Nhóm bổ sung</t>
         </is>
@@ -12271,7 +13530,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -12297,7 +13556,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="C3" s="55" t="inlineStr">
+      <c r="C3" s="59" t="inlineStr">
         <is>
           <t>TÁC ĐỘNG →</t>
         </is>
@@ -12329,23 +13588,23 @@
       <c r="B5" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="C5" s="56">
+      <c r="C5" s="60">
         <f>TRIM(IF(AND(RuiRo!$F$5=5,RuiRo!$G$5=1),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=5,RuiRo!$G$6=1),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=5,RuiRo!$G$7=1),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=5,RuiRo!$G$8=1),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=5,RuiRo!$G$9=1),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=5,RuiRo!$G$10=1),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=5,RuiRo!$G$11=1),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=5,RuiRo!$G$12=1),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=5,RuiRo!$G$13=1),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=5,RuiRo!$G$14=1),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=5,RuiRo!$G$15=1),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=5,RuiRo!$G$16=1),RuiRo!$A$16&amp;" ",""))</f>
         <v/>
       </c>
-      <c r="D5" s="57">
+      <c r="D5" s="61">
         <f>TRIM(IF(AND(RuiRo!$F$5=5,RuiRo!$G$5=2),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=5,RuiRo!$G$6=2),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=5,RuiRo!$G$7=2),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=5,RuiRo!$G$8=2),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=5,RuiRo!$G$9=2),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=5,RuiRo!$G$10=2),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=5,RuiRo!$G$11=2),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=5,RuiRo!$G$12=2),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=5,RuiRo!$G$13=2),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=5,RuiRo!$G$14=2),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=5,RuiRo!$G$15=2),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=5,RuiRo!$G$16=2),RuiRo!$A$16&amp;" ",""))</f>
         <v/>
       </c>
-      <c r="E5" s="58">
+      <c r="E5" s="62">
         <f>TRIM(IF(AND(RuiRo!$F$5=5,RuiRo!$G$5=3),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=5,RuiRo!$G$6=3),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=5,RuiRo!$G$7=3),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=5,RuiRo!$G$8=3),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=5,RuiRo!$G$9=3),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=5,RuiRo!$G$10=3),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=5,RuiRo!$G$11=3),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=5,RuiRo!$G$12=3),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=5,RuiRo!$G$13=3),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=5,RuiRo!$G$14=3),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=5,RuiRo!$G$15=3),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=5,RuiRo!$G$16=3),RuiRo!$A$16&amp;" ",""))</f>
         <v/>
       </c>
-      <c r="F5" s="58">
+      <c r="F5" s="62">
         <f>TRIM(IF(AND(RuiRo!$F$5=5,RuiRo!$G$5=4),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=5,RuiRo!$G$6=4),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=5,RuiRo!$G$7=4),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=5,RuiRo!$G$8=4),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=5,RuiRo!$G$9=4),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=5,RuiRo!$G$10=4),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=5,RuiRo!$G$11=4),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=5,RuiRo!$G$12=4),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=5,RuiRo!$G$13=4),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=5,RuiRo!$G$14=4),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=5,RuiRo!$G$15=4),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=5,RuiRo!$G$16=4),RuiRo!$A$16&amp;" ",""))</f>
         <v/>
       </c>
-      <c r="G5" s="58">
+      <c r="G5" s="62">
         <f>TRIM(IF(AND(RuiRo!$F$5=5,RuiRo!$G$5=5),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=5,RuiRo!$G$6=5),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=5,RuiRo!$G$7=5),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=5,RuiRo!$G$8=5),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=5,RuiRo!$G$9=5),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=5,RuiRo!$G$10=5),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=5,RuiRo!$G$11=5),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=5,RuiRo!$G$12=5),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=5,RuiRo!$G$13=5),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=5,RuiRo!$G$14=5),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=5,RuiRo!$G$15=5),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=5,RuiRo!$G$16=5),RuiRo!$A$16&amp;" ",""))</f>
         <v/>
       </c>
@@ -12354,23 +13613,23 @@
       <c r="B6" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="C6" s="56">
+      <c r="C6" s="60">
         <f>TRIM(IF(AND(RuiRo!$F$5=4,RuiRo!$G$5=1),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=4,RuiRo!$G$6=1),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=4,RuiRo!$G$7=1),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=4,RuiRo!$G$8=1),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=4,RuiRo!$G$9=1),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=4,RuiRo!$G$10=1),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=4,RuiRo!$G$11=1),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=4,RuiRo!$G$12=1),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=4,RuiRo!$G$13=1),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=4,RuiRo!$G$14=1),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=4,RuiRo!$G$15=1),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=4,RuiRo!$G$16=1),RuiRo!$A$16&amp;" ",""))</f>
         <v/>
       </c>
-      <c r="D6" s="57">
+      <c r="D6" s="61">
         <f>TRIM(IF(AND(RuiRo!$F$5=4,RuiRo!$G$5=2),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=4,RuiRo!$G$6=2),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=4,RuiRo!$G$7=2),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=4,RuiRo!$G$8=2),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=4,RuiRo!$G$9=2),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=4,RuiRo!$G$10=2),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=4,RuiRo!$G$11=2),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=4,RuiRo!$G$12=2),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=4,RuiRo!$G$13=2),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=4,RuiRo!$G$14=2),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=4,RuiRo!$G$15=2),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=4,RuiRo!$G$16=2),RuiRo!$A$16&amp;" ",""))</f>
         <v/>
       </c>
-      <c r="E6" s="57">
+      <c r="E6" s="61">
         <f>TRIM(IF(AND(RuiRo!$F$5=4,RuiRo!$G$5=3),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=4,RuiRo!$G$6=3),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=4,RuiRo!$G$7=3),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=4,RuiRo!$G$8=3),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=4,RuiRo!$G$9=3),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=4,RuiRo!$G$10=3),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=4,RuiRo!$G$11=3),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=4,RuiRo!$G$12=3),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=4,RuiRo!$G$13=3),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=4,RuiRo!$G$14=3),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=4,RuiRo!$G$15=3),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=4,RuiRo!$G$16=3),RuiRo!$A$16&amp;" ",""))</f>
         <v/>
       </c>
-      <c r="F6" s="58">
+      <c r="F6" s="62">
         <f>TRIM(IF(AND(RuiRo!$F$5=4,RuiRo!$G$5=4),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=4,RuiRo!$G$6=4),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=4,RuiRo!$G$7=4),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=4,RuiRo!$G$8=4),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=4,RuiRo!$G$9=4),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=4,RuiRo!$G$10=4),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=4,RuiRo!$G$11=4),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=4,RuiRo!$G$12=4),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=4,RuiRo!$G$13=4),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=4,RuiRo!$G$14=4),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=4,RuiRo!$G$15=4),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=4,RuiRo!$G$16=4),RuiRo!$A$16&amp;" ",""))</f>
         <v/>
       </c>
-      <c r="G6" s="58">
+      <c r="G6" s="62">
         <f>TRIM(IF(AND(RuiRo!$F$5=4,RuiRo!$G$5=5),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=4,RuiRo!$G$6=5),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=4,RuiRo!$G$7=5),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=4,RuiRo!$G$8=5),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=4,RuiRo!$G$9=5),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=4,RuiRo!$G$10=5),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=4,RuiRo!$G$11=5),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=4,RuiRo!$G$12=5),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=4,RuiRo!$G$13=5),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=4,RuiRo!$G$14=5),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=4,RuiRo!$G$15=5),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=4,RuiRo!$G$16=5),RuiRo!$A$16&amp;" ",""))</f>
         <v/>
       </c>
@@ -12379,23 +13638,23 @@
       <c r="B7" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="C7" s="56">
+      <c r="C7" s="60">
         <f>TRIM(IF(AND(RuiRo!$F$5=3,RuiRo!$G$5=1),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=3,RuiRo!$G$6=1),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=3,RuiRo!$G$7=1),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=3,RuiRo!$G$8=1),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=3,RuiRo!$G$9=1),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=3,RuiRo!$G$10=1),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=3,RuiRo!$G$11=1),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=3,RuiRo!$G$12=1),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=3,RuiRo!$G$13=1),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=3,RuiRo!$G$14=1),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=3,RuiRo!$G$15=1),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=3,RuiRo!$G$16=1),RuiRo!$A$16&amp;" ",""))</f>
         <v/>
       </c>
-      <c r="D7" s="56">
+      <c r="D7" s="60">
         <f>TRIM(IF(AND(RuiRo!$F$5=3,RuiRo!$G$5=2),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=3,RuiRo!$G$6=2),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=3,RuiRo!$G$7=2),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=3,RuiRo!$G$8=2),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=3,RuiRo!$G$9=2),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=3,RuiRo!$G$10=2),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=3,RuiRo!$G$11=2),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=3,RuiRo!$G$12=2),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=3,RuiRo!$G$13=2),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=3,RuiRo!$G$14=2),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=3,RuiRo!$G$15=2),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=3,RuiRo!$G$16=2),RuiRo!$A$16&amp;" ",""))</f>
         <v/>
       </c>
-      <c r="E7" s="57">
+      <c r="E7" s="61">
         <f>TRIM(IF(AND(RuiRo!$F$5=3,RuiRo!$G$5=3),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=3,RuiRo!$G$6=3),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=3,RuiRo!$G$7=3),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=3,RuiRo!$G$8=3),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=3,RuiRo!$G$9=3),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=3,RuiRo!$G$10=3),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=3,RuiRo!$G$11=3),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=3,RuiRo!$G$12=3),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=3,RuiRo!$G$13=3),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=3,RuiRo!$G$14=3),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=3,RuiRo!$G$15=3),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=3,RuiRo!$G$16=3),RuiRo!$A$16&amp;" ",""))</f>
         <v/>
       </c>
-      <c r="F7" s="57">
+      <c r="F7" s="61">
         <f>TRIM(IF(AND(RuiRo!$F$5=3,RuiRo!$G$5=4),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=3,RuiRo!$G$6=4),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=3,RuiRo!$G$7=4),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=3,RuiRo!$G$8=4),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=3,RuiRo!$G$9=4),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=3,RuiRo!$G$10=4),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=3,RuiRo!$G$11=4),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=3,RuiRo!$G$12=4),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=3,RuiRo!$G$13=4),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=3,RuiRo!$G$14=4),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=3,RuiRo!$G$15=4),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=3,RuiRo!$G$16=4),RuiRo!$A$16&amp;" ",""))</f>
         <v/>
       </c>
-      <c r="G7" s="58">
+      <c r="G7" s="62">
         <f>TRIM(IF(AND(RuiRo!$F$5=3,RuiRo!$G$5=5),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=3,RuiRo!$G$6=5),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=3,RuiRo!$G$7=5),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=3,RuiRo!$G$8=5),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=3,RuiRo!$G$9=5),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=3,RuiRo!$G$10=5),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=3,RuiRo!$G$11=5),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=3,RuiRo!$G$12=5),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=3,RuiRo!$G$13=5),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=3,RuiRo!$G$14=5),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=3,RuiRo!$G$15=5),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=3,RuiRo!$G$16=5),RuiRo!$A$16&amp;" ",""))</f>
         <v/>
       </c>
@@ -12404,23 +13663,23 @@
       <c r="B8" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="C8" s="56">
+      <c r="C8" s="60">
         <f>TRIM(IF(AND(RuiRo!$F$5=2,RuiRo!$G$5=1),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=2,RuiRo!$G$6=1),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=2,RuiRo!$G$7=1),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=2,RuiRo!$G$8=1),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=2,RuiRo!$G$9=1),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=2,RuiRo!$G$10=1),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=2,RuiRo!$G$11=1),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=2,RuiRo!$G$12=1),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=2,RuiRo!$G$13=1),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=2,RuiRo!$G$14=1),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=2,RuiRo!$G$15=1),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=2,RuiRo!$G$16=1),RuiRo!$A$16&amp;" ",""))</f>
         <v/>
       </c>
-      <c r="D8" s="56">
+      <c r="D8" s="60">
         <f>TRIM(IF(AND(RuiRo!$F$5=2,RuiRo!$G$5=2),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=2,RuiRo!$G$6=2),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=2,RuiRo!$G$7=2),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=2,RuiRo!$G$8=2),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=2,RuiRo!$G$9=2),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=2,RuiRo!$G$10=2),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=2,RuiRo!$G$11=2),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=2,RuiRo!$G$12=2),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=2,RuiRo!$G$13=2),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=2,RuiRo!$G$14=2),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=2,RuiRo!$G$15=2),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=2,RuiRo!$G$16=2),RuiRo!$A$16&amp;" ",""))</f>
         <v/>
       </c>
-      <c r="E8" s="56">
+      <c r="E8" s="60">
         <f>TRIM(IF(AND(RuiRo!$F$5=2,RuiRo!$G$5=3),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=2,RuiRo!$G$6=3),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=2,RuiRo!$G$7=3),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=2,RuiRo!$G$8=3),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=2,RuiRo!$G$9=3),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=2,RuiRo!$G$10=3),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=2,RuiRo!$G$11=3),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=2,RuiRo!$G$12=3),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=2,RuiRo!$G$13=3),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=2,RuiRo!$G$14=3),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=2,RuiRo!$G$15=3),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=2,RuiRo!$G$16=3),RuiRo!$A$16&amp;" ",""))</f>
         <v/>
       </c>
-      <c r="F8" s="57">
+      <c r="F8" s="61">
         <f>TRIM(IF(AND(RuiRo!$F$5=2,RuiRo!$G$5=4),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=2,RuiRo!$G$6=4),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=2,RuiRo!$G$7=4),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=2,RuiRo!$G$8=4),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=2,RuiRo!$G$9=4),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=2,RuiRo!$G$10=4),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=2,RuiRo!$G$11=4),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=2,RuiRo!$G$12=4),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=2,RuiRo!$G$13=4),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=2,RuiRo!$G$14=4),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=2,RuiRo!$G$15=4),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=2,RuiRo!$G$16=4),RuiRo!$A$16&amp;" ",""))</f>
         <v/>
       </c>
-      <c r="G8" s="57">
+      <c r="G8" s="61">
         <f>TRIM(IF(AND(RuiRo!$F$5=2,RuiRo!$G$5=5),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=2,RuiRo!$G$6=5),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=2,RuiRo!$G$7=5),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=2,RuiRo!$G$8=5),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=2,RuiRo!$G$9=5),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=2,RuiRo!$G$10=5),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=2,RuiRo!$G$11=5),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=2,RuiRo!$G$12=5),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=2,RuiRo!$G$13=5),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=2,RuiRo!$G$14=5),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=2,RuiRo!$G$15=5),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=2,RuiRo!$G$16=5),RuiRo!$A$16&amp;" ",""))</f>
         <v/>
       </c>
@@ -12429,23 +13688,23 @@
       <c r="B9" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="C9" s="56">
+      <c r="C9" s="60">
         <f>TRIM(IF(AND(RuiRo!$F$5=1,RuiRo!$G$5=1),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=1,RuiRo!$G$6=1),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=1,RuiRo!$G$7=1),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=1,RuiRo!$G$8=1),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=1,RuiRo!$G$9=1),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=1,RuiRo!$G$10=1),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=1,RuiRo!$G$11=1),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=1,RuiRo!$G$12=1),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=1,RuiRo!$G$13=1),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=1,RuiRo!$G$14=1),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=1,RuiRo!$G$15=1),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=1,RuiRo!$G$16=1),RuiRo!$A$16&amp;" ",""))</f>
         <v/>
       </c>
-      <c r="D9" s="56">
+      <c r="D9" s="60">
         <f>TRIM(IF(AND(RuiRo!$F$5=1,RuiRo!$G$5=2),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=1,RuiRo!$G$6=2),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=1,RuiRo!$G$7=2),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=1,RuiRo!$G$8=2),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=1,RuiRo!$G$9=2),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=1,RuiRo!$G$10=2),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=1,RuiRo!$G$11=2),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=1,RuiRo!$G$12=2),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=1,RuiRo!$G$13=2),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=1,RuiRo!$G$14=2),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=1,RuiRo!$G$15=2),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=1,RuiRo!$G$16=2),RuiRo!$A$16&amp;" ",""))</f>
         <v/>
       </c>
-      <c r="E9" s="56">
+      <c r="E9" s="60">
         <f>TRIM(IF(AND(RuiRo!$F$5=1,RuiRo!$G$5=3),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=1,RuiRo!$G$6=3),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=1,RuiRo!$G$7=3),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=1,RuiRo!$G$8=3),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=1,RuiRo!$G$9=3),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=1,RuiRo!$G$10=3),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=1,RuiRo!$G$11=3),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=1,RuiRo!$G$12=3),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=1,RuiRo!$G$13=3),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=1,RuiRo!$G$14=3),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=1,RuiRo!$G$15=3),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=1,RuiRo!$G$16=3),RuiRo!$A$16&amp;" ",""))</f>
         <v/>
       </c>
-      <c r="F9" s="56">
+      <c r="F9" s="60">
         <f>TRIM(IF(AND(RuiRo!$F$5=1,RuiRo!$G$5=4),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=1,RuiRo!$G$6=4),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=1,RuiRo!$G$7=4),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=1,RuiRo!$G$8=4),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=1,RuiRo!$G$9=4),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=1,RuiRo!$G$10=4),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=1,RuiRo!$G$11=4),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=1,RuiRo!$G$12=4),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=1,RuiRo!$G$13=4),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=1,RuiRo!$G$14=4),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=1,RuiRo!$G$15=4),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=1,RuiRo!$G$16=4),RuiRo!$A$16&amp;" ",""))</f>
         <v/>
       </c>
-      <c r="G9" s="56">
+      <c r="G9" s="60">
         <f>TRIM(IF(AND(RuiRo!$F$5=1,RuiRo!$G$5=5),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=1,RuiRo!$G$6=5),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=1,RuiRo!$G$7=5),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=1,RuiRo!$G$8=5),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=1,RuiRo!$G$9=5),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=1,RuiRo!$G$10=5),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=1,RuiRo!$G$11=5),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=1,RuiRo!$G$12=5),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=1,RuiRo!$G$13=5),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=1,RuiRo!$G$14=5),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=1,RuiRo!$G$15=5),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=1,RuiRo!$G$16=5),RuiRo!$A$16&amp;" ",""))</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Lab: thêm rủi ro R11 (thành viên nghỉ đột xuất vì việc gia đình) do nhóm bổ sung
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/lab/QLDA_PharmaDash_LichDuAn.xlsx
+++ b/docs/lab/QLDA_PharmaDash_LichDuAn.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\nhà thuốc\docs\lab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CBB61F0-865E-4C53-9AE4-05C5D94C7546}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22B04BB6-FCE3-4C45-9E03-FADB1624A9D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="655" uniqueCount="477">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="662" uniqueCount="481">
   <si>
     <t>LỊCH DỰ ÁN PHARMADASH – Bài Lab QLDA CNTT</t>
   </si>
@@ -1495,6 +1495,18 @@
   </si>
   <si>
     <t>Vùng đỏ: điểm ≥ 15 (Cao) · Cam: 8–14 (Trung bình) · Xanh: &lt; 8 (Thấp)</t>
+  </si>
+  <si>
+    <t>Gói việc của người đó bị dừng; nếu là việc trên đường găng (BE, FE) thì cả dự án trễ theo</t>
+  </si>
+  <si>
+    <t>Một thành viên phải nghỉ vài ngày đến 1 tuần, không báo trước được</t>
+  </si>
+  <si>
+    <t>Thành viên có việc gia đình đột xuất (đồ án trước của nhóm từng bị trễ vì lý do này)</t>
+  </si>
+  <si>
+    <t>Mỗi người có 1 "người đỡ" (buddy) nắm việc của mình; cập nhật tiến độ hằng ngày trên nhóm chat; đẩy code lên GitHub cuối mỗi ngày để người khác làm tiếp được</t>
   </si>
 </sst>
 </file>
@@ -1504,12 +1516,12 @@
   <numFmts count="6">
     <numFmt numFmtId="164" formatCode="#,##0;\(#,##0\);\-"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
-    <numFmt numFmtId="167" formatCode="dd/mm/yyyy"/>
-    <numFmt numFmtId="168" formatCode="dd/mm"/>
-    <numFmt numFmtId="169" formatCode="0.0"/>
-    <numFmt numFmtId="170" formatCode=";;;"/>
+    <numFmt numFmtId="166" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="167" formatCode="dd/mm"/>
+    <numFmt numFmtId="168" formatCode="0.0"/>
+    <numFmt numFmtId="169" formatCode=";;;"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1570,6 +1582,11 @@
       <color indexed="81"/>
       <name val="Tahoma"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="10">
@@ -1686,7 +1703,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1749,25 +1766,25 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="169" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="6" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="6" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="6" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1791,15 +1808,22 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -5681,7 +5705,7 @@
       <c r="A26" s="59" t="s">
         <v>359</v>
       </c>
-      <c r="B26" s="60"/>
+      <c r="B26" s="62"/>
       <c r="C26" s="41">
         <f>MAX(L9:L23)</f>
         <v>75.333333333333329</v>
@@ -5691,24 +5715,24 @@
       <c r="A27" s="59" t="s">
         <v>360</v>
       </c>
-      <c r="B27" s="60"/>
+      <c r="B27" s="62"/>
       <c r="C27" s="59" t="str">
         <f>LEFT(IF(P9="Găng","A → ","")&amp;IF(P10="Găng","B → ","")&amp;IF(P11="Găng","C → ","")&amp;IF(P12="Găng","D → ","")&amp;IF(P13="Găng","E → ","")&amp;IF(P14="Găng","F → ","")&amp;IF(P15="Găng","G → ","")&amp;IF(P16="Găng","H → ","")&amp;IF(P17="Găng","I → ","")&amp;IF(P18="Găng","J → ","")&amp;IF(P19="Găng","K → ","")&amp;IF(P20="Găng","L → ","")&amp;IF(P21="Găng","M → ","")&amp;IF(P22="Găng","N → ","")&amp;IF(P23="Găng","O → ",""),LEN(IF(P9="Găng","A → ","")&amp;IF(P10="Găng","B → ","")&amp;IF(P11="Găng","C → ","")&amp;IF(P12="Găng","D → ","")&amp;IF(P13="Găng","E → ","")&amp;IF(P14="Găng","F → ","")&amp;IF(P15="Găng","G → ","")&amp;IF(P16="Găng","H → ","")&amp;IF(P17="Găng","I → ","")&amp;IF(P18="Găng","J → ","")&amp;IF(P19="Găng","K → ","")&amp;IF(P20="Găng","L → ","")&amp;IF(P21="Găng","M → ","")&amp;IF(P22="Găng","N → ","")&amp;IF(P23="Găng","O → ",""))-3)</f>
         <v>A → B → C → E → I → J → M → N → O</v>
       </c>
-      <c r="D27" s="61"/>
-      <c r="E27" s="61"/>
-      <c r="F27" s="61"/>
-      <c r="G27" s="61"/>
-      <c r="H27" s="61"/>
-      <c r="I27" s="61"/>
-      <c r="J27" s="62"/>
+      <c r="D27" s="60"/>
+      <c r="E27" s="60"/>
+      <c r="F27" s="60"/>
+      <c r="G27" s="60"/>
+      <c r="H27" s="60"/>
+      <c r="I27" s="60"/>
+      <c r="J27" s="61"/>
     </row>
     <row r="28" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A28" s="59" t="s">
         <v>361</v>
       </c>
-      <c r="B28" s="60"/>
+      <c r="B28" s="62"/>
       <c r="C28" s="41">
         <f>SUMIF(P9:P23,"Găng",J9:J23)</f>
         <v>13.055555555555557</v>
@@ -5718,7 +5742,7 @@
       <c r="A29" s="59" t="s">
         <v>362</v>
       </c>
-      <c r="B29" s="60"/>
+      <c r="B29" s="62"/>
       <c r="C29" s="41">
         <f>SQRT(C28)</f>
         <v>3.6132472314464668</v>
@@ -5728,7 +5752,7 @@
       <c r="A30" s="59" t="s">
         <v>363</v>
       </c>
-      <c r="B30" s="60"/>
+      <c r="B30" s="62"/>
       <c r="C30" s="29">
         <f>C5</f>
         <v>64</v>
@@ -5738,7 +5762,7 @@
       <c r="A31" s="59" t="s">
         <v>364</v>
       </c>
-      <c r="B31" s="60"/>
+      <c r="B31" s="62"/>
       <c r="C31" s="41">
         <f>C26-C30</f>
         <v>11.333333333333329</v>
@@ -5748,7 +5772,7 @@
       <c r="A32" s="59" t="s">
         <v>365</v>
       </c>
-      <c r="B32" s="60"/>
+      <c r="B32" s="62"/>
       <c r="C32" s="41">
         <f>(C30-C26)/C29</f>
         <v>-3.1366061072982077</v>
@@ -5758,7 +5782,7 @@
       <c r="A33" s="59" t="s">
         <v>366</v>
       </c>
-      <c r="B33" s="60"/>
+      <c r="B33" s="62"/>
       <c r="C33" s="42">
         <f>NORMSDIST(C32)</f>
         <v>8.5457789242917941E-4</v>
@@ -5768,7 +5792,7 @@
       <c r="A34" s="59" t="s">
         <v>367</v>
       </c>
-      <c r="B34" s="60"/>
+      <c r="B34" s="62"/>
       <c r="C34" s="43">
         <f>WORKDAY(C3,ROUNDUP(C26,0)-1)</f>
         <v>46405</v>
@@ -5778,7 +5802,7 @@
       <c r="A35" s="59" t="s">
         <v>298</v>
       </c>
-      <c r="B35" s="60"/>
+      <c r="B35" s="62"/>
       <c r="C35" s="26" t="str">
         <f>IF(C31&lt;=0,"Kịp hạn chót","TRỄ HẠN – cần nén lịch (crashing / fast-tracking)")</f>
         <v>TRỄ HẠN – cần nén lịch (crashing / fast-tracking)</v>
@@ -5786,17 +5810,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="C27:J27"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="A31:B31"/>
-    <mergeCell ref="A34:B34"/>
-    <mergeCell ref="A35:B35"/>
     <mergeCell ref="A26:B26"/>
     <mergeCell ref="A30:B30"/>
     <mergeCell ref="A29:B29"/>
     <mergeCell ref="A33:B33"/>
     <mergeCell ref="A28:B28"/>
     <mergeCell ref="A32:B32"/>
+    <mergeCell ref="C27:J27"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="A35:B35"/>
   </mergeCells>
   <conditionalFormatting sqref="A9:P23">
     <cfRule type="expression" dxfId="8" priority="1">
@@ -12010,7 +12034,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:16" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A5" s="28" t="s">
         <v>324</v>
       </c>
@@ -12314,7 +12338,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:16" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A10" s="28" t="s">
         <v>336</v>
       </c>
@@ -12433,7 +12457,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:16" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A12" s="28" t="s">
         <v>340</v>
       </c>
@@ -12925,7 +12949,7 @@
       <c r="A22" s="59" t="s">
         <v>383</v>
       </c>
-      <c r="B22" s="60"/>
+      <c r="B22" s="62"/>
       <c r="C22" s="41">
         <f>MAX(K5:K19)</f>
         <v>61.833333333333336</v>
@@ -12935,24 +12959,24 @@
       <c r="A23" s="59" t="s">
         <v>384</v>
       </c>
-      <c r="B23" s="60"/>
+      <c r="B23" s="62"/>
       <c r="C23" s="59" t="str">
         <f>LEFT(IF(O5="Găng","A → ","")&amp;IF(O6="Găng","B → ","")&amp;IF(O7="Găng","C → ","")&amp;IF(O8="Găng","D → ","")&amp;IF(O9="Găng","E → ","")&amp;IF(O10="Găng","F → ","")&amp;IF(O11="Găng","G → ","")&amp;IF(O12="Găng","H → ","")&amp;IF(O13="Găng","I → ","")&amp;IF(O14="Găng","J → ","")&amp;IF(O15="Găng","K → ","")&amp;IF(O16="Găng","L → ","")&amp;IF(O17="Găng","M → ","")&amp;IF(O18="Găng","N → ","")&amp;IF(O19="Găng","O → ",""),LEN(IF(O5="Găng","A → ","")&amp;IF(O6="Găng","B → ","")&amp;IF(O7="Găng","C → ","")&amp;IF(O8="Găng","D → ","")&amp;IF(O9="Găng","E → ","")&amp;IF(O10="Găng","F → ","")&amp;IF(O11="Găng","G → ","")&amp;IF(O12="Găng","H → ","")&amp;IF(O13="Găng","I → ","")&amp;IF(O14="Găng","J → ","")&amp;IF(O15="Găng","K → ","")&amp;IF(O16="Găng","L → ","")&amp;IF(O17="Găng","M → ","")&amp;IF(O18="Găng","N → ","")&amp;IF(O19="Găng","O → ",""))-3)</f>
         <v>A → B → C → D → F → G → K → M → N → O</v>
       </c>
-      <c r="D23" s="61"/>
-      <c r="E23" s="61"/>
-      <c r="F23" s="61"/>
-      <c r="G23" s="61"/>
-      <c r="H23" s="61"/>
-      <c r="I23" s="61"/>
-      <c r="J23" s="62"/>
+      <c r="D23" s="60"/>
+      <c r="E23" s="60"/>
+      <c r="F23" s="60"/>
+      <c r="G23" s="60"/>
+      <c r="H23" s="60"/>
+      <c r="I23" s="60"/>
+      <c r="J23" s="61"/>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A24" s="59" t="s">
         <v>362</v>
       </c>
-      <c r="B24" s="60"/>
+      <c r="B24" s="62"/>
       <c r="C24" s="41">
         <f>SQRT(SUMIF(O5:O19,"Găng",I5:I19))</f>
         <v>3.3870669054835965</v>
@@ -12962,7 +12986,7 @@
       <c r="A25" s="59" t="s">
         <v>363</v>
       </c>
-      <c r="B25" s="60"/>
+      <c r="B25" s="62"/>
       <c r="C25" s="29">
         <f>PERT!C5</f>
         <v>64</v>
@@ -12972,7 +12996,7 @@
       <c r="A26" s="59" t="s">
         <v>385</v>
       </c>
-      <c r="B26" s="60"/>
+      <c r="B26" s="62"/>
       <c r="C26" s="41">
         <f>C25-C22</f>
         <v>2.1666666666666643</v>
@@ -12982,7 +13006,7 @@
       <c r="A27" s="59" t="s">
         <v>386</v>
       </c>
-      <c r="B27" s="60"/>
+      <c r="B27" s="62"/>
       <c r="C27" s="35">
         <f>NORMSDIST((C25-C22)/C24)</f>
         <v>0.73881232950538911</v>
@@ -12992,7 +13016,7 @@
       <c r="A28" s="59" t="s">
         <v>387</v>
       </c>
-      <c r="B28" s="60"/>
+      <c r="B28" s="62"/>
       <c r="C28" s="43">
         <f>WORKDAY(PERT!C3,ROUNDUP(C22,0)-1)</f>
         <v>46385</v>
@@ -13002,7 +13026,7 @@
       <c r="A29" s="59" t="s">
         <v>388</v>
       </c>
-      <c r="B29" s="60"/>
+      <c r="B29" s="62"/>
       <c r="C29" s="41">
         <f>PERT!$C$26</f>
         <v>75.333333333333329</v>
@@ -13014,6 +13038,9 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="A28:B28"/>
     <mergeCell ref="A23:B23"/>
     <mergeCell ref="A27:B27"/>
     <mergeCell ref="C23:J23"/>
@@ -13021,9 +13048,6 @@
     <mergeCell ref="A2:P2"/>
     <mergeCell ref="A26:B26"/>
     <mergeCell ref="A24:B24"/>
-    <mergeCell ref="A29:B29"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="A28:B28"/>
   </mergeCells>
   <conditionalFormatting sqref="A5:O19">
     <cfRule type="expression" dxfId="3" priority="1">
@@ -13124,11 +13148,11 @@
         <v>5</v>
       </c>
       <c r="H5" s="54">
-        <f t="shared" ref="H5:H14" si="0">F5*G5</f>
+        <f>F5*G5</f>
         <v>20</v>
       </c>
       <c r="I5" s="28" t="str">
-        <f t="shared" ref="I5:I14" si="1">IF(H5&gt;=15,"Cao",IF(H5&gt;=8,"Trung bình","Thấp"))</f>
+        <f>IF(H5&gt;=15,"Cao",IF(H5&gt;=8,"Trung bình","Thấp"))</f>
         <v>Cao</v>
       </c>
       <c r="J5" s="24" t="s">
@@ -13167,11 +13191,11 @@
         <v>4</v>
       </c>
       <c r="H6" s="54">
-        <f t="shared" si="0"/>
+        <f>F6*G6</f>
         <v>16</v>
       </c>
       <c r="I6" s="28" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(H6&gt;=15,"Cao",IF(H6&gt;=8,"Trung bình","Thấp"))</f>
         <v>Cao</v>
       </c>
       <c r="J6" s="24" t="s">
@@ -13210,11 +13234,11 @@
         <v>4</v>
       </c>
       <c r="H7" s="54">
-        <f t="shared" si="0"/>
+        <f>F7*G7</f>
         <v>16</v>
       </c>
       <c r="I7" s="28" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(H7&gt;=15,"Cao",IF(H7&gt;=8,"Trung bình","Thấp"))</f>
         <v>Cao</v>
       </c>
       <c r="J7" s="24" t="s">
@@ -13253,11 +13277,11 @@
         <v>4</v>
       </c>
       <c r="H8" s="54">
-        <f t="shared" si="0"/>
+        <f>F8*G8</f>
         <v>16</v>
       </c>
       <c r="I8" s="28" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(H8&gt;=15,"Cao",IF(H8&gt;=8,"Trung bình","Thấp"))</f>
         <v>Cao</v>
       </c>
       <c r="J8" s="24" t="s">
@@ -13296,11 +13320,11 @@
         <v>5</v>
       </c>
       <c r="H9" s="54">
-        <f t="shared" si="0"/>
+        <f>F9*G9</f>
         <v>15</v>
       </c>
       <c r="I9" s="28" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(H9&gt;=15,"Cao",IF(H9&gt;=8,"Trung bình","Thấp"))</f>
         <v>Cao</v>
       </c>
       <c r="J9" s="24" t="s">
@@ -13316,87 +13340,87 @@
         <v>412</v>
       </c>
     </row>
-    <row r="10" spans="1:13" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A10" s="52" t="s">
-        <v>438</v>
-      </c>
-      <c r="B10" s="24" t="s">
-        <v>439</v>
-      </c>
-      <c r="C10" s="24" t="s">
-        <v>440</v>
-      </c>
-      <c r="D10" s="24" t="s">
-        <v>441</v>
-      </c>
-      <c r="E10" s="24" t="s">
-        <v>442</v>
-      </c>
-      <c r="F10" s="53">
-        <v>2</v>
-      </c>
-      <c r="G10" s="53">
-        <v>5</v>
-      </c>
-      <c r="H10" s="54">
-        <f t="shared" si="0"/>
-        <v>10</v>
-      </c>
-      <c r="I10" s="28" t="str">
-        <f t="shared" si="1"/>
+    <row r="10" spans="1:13" ht="52.8" x14ac:dyDescent="0.3">
+      <c r="A10" s="66" t="s">
+        <v>470</v>
+      </c>
+      <c r="B10" s="68" t="s">
+        <v>479</v>
+      </c>
+      <c r="C10" s="68" t="s">
+        <v>478</v>
+      </c>
+      <c r="D10" s="68" t="s">
+        <v>477</v>
+      </c>
+      <c r="E10" s="68" t="s">
+        <v>436</v>
+      </c>
+      <c r="F10" s="67">
+        <v>3</v>
+      </c>
+      <c r="G10" s="67">
+        <v>4</v>
+      </c>
+      <c r="H10" s="67">
+        <f>IF(OR(F10="",G10=""),"",F10*G10)</f>
+        <v>12</v>
+      </c>
+      <c r="I10" s="67" t="str">
+        <f>IF(H10="","",IF(H10&gt;=15,"Cao",IF(H10&gt;=8,"Trung bình","Thấp")))</f>
         <v>Trung bình</v>
       </c>
-      <c r="J10" s="24" t="s">
+      <c r="J10" s="68" t="s">
         <v>409</v>
       </c>
-      <c r="K10" s="24" t="s">
-        <v>443</v>
-      </c>
-      <c r="L10" s="24" t="s">
-        <v>444</v>
-      </c>
-      <c r="M10" s="23" t="s">
-        <v>412</v>
+      <c r="K10" s="68" t="s">
+        <v>480</v>
+      </c>
+      <c r="L10" s="68" t="s">
+        <v>40</v>
+      </c>
+      <c r="M10" s="67" t="s">
+        <v>471</v>
       </c>
     </row>
     <row r="11" spans="1:13" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A11" s="52" t="s">
-        <v>445</v>
+        <v>438</v>
       </c>
       <c r="B11" s="24" t="s">
-        <v>446</v>
+        <v>439</v>
       </c>
       <c r="C11" s="24" t="s">
-        <v>447</v>
+        <v>440</v>
       </c>
       <c r="D11" s="24" t="s">
-        <v>448</v>
+        <v>441</v>
       </c>
       <c r="E11" s="24" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="F11" s="53">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G11" s="53">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H11" s="54">
-        <f t="shared" si="0"/>
-        <v>9</v>
+        <f>F11*G11</f>
+        <v>10</v>
       </c>
       <c r="I11" s="28" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(H11&gt;=15,"Cao",IF(H11&gt;=8,"Trung bình","Thấp"))</f>
         <v>Trung bình</v>
       </c>
       <c r="J11" s="24" t="s">
         <v>409</v>
       </c>
       <c r="K11" s="24" t="s">
-        <v>450</v>
+        <v>443</v>
       </c>
       <c r="L11" s="24" t="s">
-        <v>80</v>
+        <v>444</v>
       </c>
       <c r="M11" s="23" t="s">
         <v>412</v>
@@ -13404,19 +13428,19 @@
     </row>
     <row r="12" spans="1:13" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A12" s="52" t="s">
-        <v>451</v>
+        <v>445</v>
       </c>
       <c r="B12" s="24" t="s">
-        <v>452</v>
+        <v>446</v>
       </c>
       <c r="C12" s="24" t="s">
-        <v>453</v>
+        <v>447</v>
       </c>
       <c r="D12" s="24" t="s">
-        <v>454</v>
+        <v>448</v>
       </c>
       <c r="E12" s="24" t="s">
-        <v>455</v>
+        <v>449</v>
       </c>
       <c r="F12" s="53">
         <v>3</v>
@@ -13425,135 +13449,153 @@
         <v>3</v>
       </c>
       <c r="H12" s="54">
-        <f t="shared" si="0"/>
+        <f>F12*G12</f>
         <v>9</v>
       </c>
       <c r="I12" s="28" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(H12&gt;=15,"Cao",IF(H12&gt;=8,"Trung bình","Thấp"))</f>
         <v>Trung bình</v>
       </c>
       <c r="J12" s="24" t="s">
         <v>409</v>
       </c>
       <c r="K12" s="24" t="s">
-        <v>456</v>
+        <v>450</v>
       </c>
       <c r="L12" s="24" t="s">
-        <v>105</v>
+        <v>80</v>
       </c>
       <c r="M12" s="23" t="s">
         <v>412</v>
       </c>
     </row>
-    <row r="13" spans="1:13" ht="52.8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:13" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A13" s="52" t="s">
-        <v>457</v>
+        <v>451</v>
       </c>
       <c r="B13" s="24" t="s">
-        <v>458</v>
+        <v>452</v>
       </c>
       <c r="C13" s="24" t="s">
-        <v>459</v>
+        <v>453</v>
       </c>
       <c r="D13" s="24" t="s">
-        <v>460</v>
+        <v>454</v>
       </c>
       <c r="E13" s="24" t="s">
-        <v>461</v>
+        <v>455</v>
       </c>
       <c r="F13" s="53">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G13" s="53">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H13" s="54">
-        <f t="shared" si="0"/>
-        <v>8</v>
+        <f>F13*G13</f>
+        <v>9</v>
       </c>
       <c r="I13" s="28" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(H13&gt;=15,"Cao",IF(H13&gt;=8,"Trung bình","Thấp"))</f>
         <v>Trung bình</v>
       </c>
       <c r="J13" s="24" t="s">
         <v>409</v>
       </c>
       <c r="K13" s="24" t="s">
-        <v>462</v>
+        <v>456</v>
       </c>
       <c r="L13" s="24" t="s">
-        <v>80</v>
+        <v>105</v>
       </c>
       <c r="M13" s="23" t="s">
         <v>412</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A14" s="52" t="s">
-        <v>463</v>
+        <v>457</v>
       </c>
       <c r="B14" s="24" t="s">
-        <v>464</v>
+        <v>458</v>
       </c>
       <c r="C14" s="24" t="s">
-        <v>465</v>
+        <v>459</v>
       </c>
       <c r="D14" s="24" t="s">
-        <v>466</v>
+        <v>460</v>
       </c>
       <c r="E14" s="24" t="s">
-        <v>467</v>
+        <v>461</v>
       </c>
       <c r="F14" s="53">
         <v>2</v>
       </c>
       <c r="G14" s="53">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H14" s="54">
-        <f t="shared" si="0"/>
-        <v>6</v>
+        <f>F14*G14</f>
+        <v>8</v>
       </c>
       <c r="I14" s="28" t="str">
-        <f t="shared" si="1"/>
-        <v>Thấp</v>
+        <f>IF(H14&gt;=15,"Cao",IF(H14&gt;=8,"Trung bình","Thấp"))</f>
+        <v>Trung bình</v>
       </c>
       <c r="J14" s="24" t="s">
-        <v>468</v>
+        <v>409</v>
       </c>
       <c r="K14" s="24" t="s">
-        <v>469</v>
+        <v>462</v>
       </c>
       <c r="L14" s="24" t="s">
-        <v>105</v>
+        <v>80</v>
       </c>
       <c r="M14" s="23" t="s">
         <v>412</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="26" t="s">
-        <v>470</v>
-      </c>
-      <c r="B15" s="55"/>
-      <c r="C15" s="55"/>
-      <c r="D15" s="55"/>
-      <c r="E15" s="55"/>
-      <c r="F15" s="55"/>
-      <c r="G15" s="55"/>
-      <c r="H15" s="55" t="str">
-        <f>IF(OR(F15="",G15=""),"",F15*G15)</f>
-        <v/>
-      </c>
-      <c r="I15" s="55" t="str">
-        <f>IF(H15="","",IF(H15&gt;=15,"Cao",IF(H15&gt;=8,"Trung bình","Thấp")))</f>
-        <v/>
-      </c>
-      <c r="J15" s="55"/>
-      <c r="K15" s="55"/>
-      <c r="L15" s="55"/>
-      <c r="M15" s="55" t="s">
-        <v>471</v>
+      <c r="A15" s="52" t="s">
+        <v>463</v>
+      </c>
+      <c r="B15" s="24" t="s">
+        <v>464</v>
+      </c>
+      <c r="C15" s="24" t="s">
+        <v>465</v>
+      </c>
+      <c r="D15" s="24" t="s">
+        <v>466</v>
+      </c>
+      <c r="E15" s="24" t="s">
+        <v>467</v>
+      </c>
+      <c r="F15" s="53">
+        <v>2</v>
+      </c>
+      <c r="G15" s="53">
+        <v>3</v>
+      </c>
+      <c r="H15" s="54">
+        <f>F15*G15</f>
+        <v>6</v>
+      </c>
+      <c r="I15" s="28" t="str">
+        <f>IF(H15&gt;=15,"Cao",IF(H15&gt;=8,"Trung bình","Thấp"))</f>
+        <v>Thấp</v>
+      </c>
+      <c r="J15" s="24" t="s">
+        <v>468</v>
+      </c>
+      <c r="K15" s="24" t="s">
+        <v>469</v>
+      </c>
+      <c r="L15" s="24" t="s">
+        <v>105</v>
+      </c>
+      <c r="M15" s="23" t="s">
+        <v>412</v>
       </c>
     </row>
     <row r="16" spans="1:13" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
@@ -13582,6 +13624,9 @@
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A5:M15">
+    <sortCondition descending="1" ref="H5"/>
+  </sortState>
   <conditionalFormatting sqref="I5:I16">
     <cfRule type="expression" dxfId="2" priority="1">
       <formula>I5="Cao"</formula>
@@ -13709,7 +13754,7 @@
       </c>
       <c r="F7" s="57" t="str">
         <f>TRIM(IF(AND(RuiRo!$F$5=3,RuiRo!$G$5=4),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=3,RuiRo!$G$6=4),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=3,RuiRo!$G$7=4),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=3,RuiRo!$G$8=4),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=3,RuiRo!$G$9=4),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=3,RuiRo!$G$10=4),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=3,RuiRo!$G$11=4),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=3,RuiRo!$G$12=4),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=3,RuiRo!$G$13=4),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=3,RuiRo!$G$14=4),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=3,RuiRo!$G$15=4),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=3,RuiRo!$G$16=4),RuiRo!$A$16&amp;" ",""))</f>
-        <v/>
+        <v>R11</v>
       </c>
       <c r="G7" s="58" t="str">
         <f>TRIM(IF(AND(RuiRo!$F$5=3,RuiRo!$G$5=5),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=3,RuiRo!$G$6=5),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=3,RuiRo!$G$7=5),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=3,RuiRo!$G$8=5),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=3,RuiRo!$G$9=5),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=3,RuiRo!$G$10=5),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=3,RuiRo!$G$11=5),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=3,RuiRo!$G$12=5),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=3,RuiRo!$G$13=5),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=3,RuiRo!$G$14=5),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=3,RuiRo!$G$15=5),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=3,RuiRo!$G$16=5),RuiRo!$A$16&amp;" ",""))</f>

</xml_diff>

<commit_message>
Lab: thêm rủi ro R12 (hiểu sai yêu cầu phải làm lại) do nhóm bổ sung
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/lab/QLDA_PharmaDash_LichDuAn.xlsx
+++ b/docs/lab/QLDA_PharmaDash_LichDuAn.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\nhà thuốc\docs\lab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22B04BB6-FCE3-4C45-9E03-FADB1624A9D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C3AE40B-9E93-43A1-A886-E7437CB23D77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="662" uniqueCount="481">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="669" uniqueCount="486">
   <si>
     <t>LỊCH DỰ ÁN PHARMADASH – Bài Lab QLDA CNTT</t>
   </si>
@@ -1507,6 +1507,21 @@
   </si>
   <si>
     <t>Mỗi người có 1 "người đỡ" (buddy) nắm việc của mình; cập nhật tiến độ hằng ngày trên nhóm chat; đẩy code lên GitHub cuối mỗi ngày để người khác làm tiếp được</t>
+  </si>
+  <si>
+    <t>Yêu cầu</t>
+  </si>
+  <si>
+    <t>Phải làm lại (rework) chức năng đã xong, tốn thêm giờ công, ăn vào 2 ngày dự trữ của lịch đã nén</t>
+  </si>
+  <si>
+    <t>Hiểu sai một yêu cầu của khách hàng (ví dụ cách tính lợi nhuận, quy tắc cảnh báo hạn dùng), phát hiện muộn khi demo hoặc UAT</t>
+  </si>
+  <si>
+    <t>Nhóm đọc yêu cầu theo cách hiểu của mình, không xác nhận lại (đồ án trước nhóm từng hiểu sai yêu cầu của giảng viên và phải làm lại)</t>
+  </si>
+  <si>
+    <t>Sau mỗi buổi làm việc với khách hàng, BA gửi lại biên bản tóm tắt yêu cầu để khách xác nhận; viết tiêu chí chấp nhận cho từng FR trước khi code; demo bản nháp sớm (mockup) thay vì chờ demo cuối tháng</t>
   </si>
 </sst>
 </file>
@@ -1703,7 +1718,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1795,9 +1810,6 @@
     <xf numFmtId="1" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1807,10 +1819,16 @@
     <xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -5702,107 +5720,107 @@
       </c>
     </row>
     <row r="26" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A26" s="59" t="s">
+      <c r="A26" s="60" t="s">
         <v>359</v>
       </c>
-      <c r="B26" s="62"/>
+      <c r="B26" s="61"/>
       <c r="C26" s="41">
         <f>MAX(L9:L23)</f>
         <v>75.333333333333329</v>
       </c>
     </row>
     <row r="27" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A27" s="59" t="s">
+      <c r="A27" s="60" t="s">
         <v>360</v>
       </c>
-      <c r="B27" s="62"/>
-      <c r="C27" s="59" t="str">
+      <c r="B27" s="61"/>
+      <c r="C27" s="60" t="str">
         <f>LEFT(IF(P9="Găng","A → ","")&amp;IF(P10="Găng","B → ","")&amp;IF(P11="Găng","C → ","")&amp;IF(P12="Găng","D → ","")&amp;IF(P13="Găng","E → ","")&amp;IF(P14="Găng","F → ","")&amp;IF(P15="Găng","G → ","")&amp;IF(P16="Găng","H → ","")&amp;IF(P17="Găng","I → ","")&amp;IF(P18="Găng","J → ","")&amp;IF(P19="Găng","K → ","")&amp;IF(P20="Găng","L → ","")&amp;IF(P21="Găng","M → ","")&amp;IF(P22="Găng","N → ","")&amp;IF(P23="Găng","O → ",""),LEN(IF(P9="Găng","A → ","")&amp;IF(P10="Găng","B → ","")&amp;IF(P11="Găng","C → ","")&amp;IF(P12="Găng","D → ","")&amp;IF(P13="Găng","E → ","")&amp;IF(P14="Găng","F → ","")&amp;IF(P15="Găng","G → ","")&amp;IF(P16="Găng","H → ","")&amp;IF(P17="Găng","I → ","")&amp;IF(P18="Găng","J → ","")&amp;IF(P19="Găng","K → ","")&amp;IF(P20="Găng","L → ","")&amp;IF(P21="Găng","M → ","")&amp;IF(P22="Găng","N → ","")&amp;IF(P23="Găng","O → ",""))-3)</f>
         <v>A → B → C → E → I → J → M → N → O</v>
       </c>
-      <c r="D27" s="60"/>
-      <c r="E27" s="60"/>
-      <c r="F27" s="60"/>
-      <c r="G27" s="60"/>
-      <c r="H27" s="60"/>
-      <c r="I27" s="60"/>
-      <c r="J27" s="61"/>
+      <c r="D27" s="62"/>
+      <c r="E27" s="62"/>
+      <c r="F27" s="62"/>
+      <c r="G27" s="62"/>
+      <c r="H27" s="62"/>
+      <c r="I27" s="62"/>
+      <c r="J27" s="63"/>
     </row>
     <row r="28" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A28" s="59" t="s">
+      <c r="A28" s="60" t="s">
         <v>361</v>
       </c>
-      <c r="B28" s="62"/>
+      <c r="B28" s="61"/>
       <c r="C28" s="41">
         <f>SUMIF(P9:P23,"Găng",J9:J23)</f>
         <v>13.055555555555557</v>
       </c>
     </row>
     <row r="29" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A29" s="59" t="s">
+      <c r="A29" s="60" t="s">
         <v>362</v>
       </c>
-      <c r="B29" s="62"/>
+      <c r="B29" s="61"/>
       <c r="C29" s="41">
         <f>SQRT(C28)</f>
         <v>3.6132472314464668</v>
       </c>
     </row>
     <row r="30" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A30" s="59" t="s">
+      <c r="A30" s="60" t="s">
         <v>363</v>
       </c>
-      <c r="B30" s="62"/>
+      <c r="B30" s="61"/>
       <c r="C30" s="29">
         <f>C5</f>
         <v>64</v>
       </c>
     </row>
     <row r="31" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A31" s="59" t="s">
+      <c r="A31" s="60" t="s">
         <v>364</v>
       </c>
-      <c r="B31" s="62"/>
+      <c r="B31" s="61"/>
       <c r="C31" s="41">
         <f>C26-C30</f>
         <v>11.333333333333329</v>
       </c>
     </row>
     <row r="32" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A32" s="59" t="s">
+      <c r="A32" s="60" t="s">
         <v>365</v>
       </c>
-      <c r="B32" s="62"/>
+      <c r="B32" s="61"/>
       <c r="C32" s="41">
         <f>(C30-C26)/C29</f>
         <v>-3.1366061072982077</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A33" s="59" t="s">
+      <c r="A33" s="60" t="s">
         <v>366</v>
       </c>
-      <c r="B33" s="62"/>
+      <c r="B33" s="61"/>
       <c r="C33" s="42">
         <f>NORMSDIST(C32)</f>
         <v>8.5457789242917941E-4</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A34" s="59" t="s">
+      <c r="A34" s="60" t="s">
         <v>367</v>
       </c>
-      <c r="B34" s="62"/>
+      <c r="B34" s="61"/>
       <c r="C34" s="43">
         <f>WORKDAY(C3,ROUNDUP(C26,0)-1)</f>
         <v>46405</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A35" s="59" t="s">
+      <c r="A35" s="60" t="s">
         <v>298</v>
       </c>
-      <c r="B35" s="62"/>
+      <c r="B35" s="61"/>
       <c r="C35" s="26" t="str">
         <f>IF(C31&lt;=0,"Kịp hạn chót","TRỄ HẠN – cần nén lịch (crashing / fast-tracking)")</f>
         <v>TRỄ HẠN – cần nén lịch (crashing / fast-tracking)</v>
@@ -5810,17 +5828,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="C27:J27"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="A35:B35"/>
     <mergeCell ref="A26:B26"/>
     <mergeCell ref="A30:B30"/>
     <mergeCell ref="A29:B29"/>
     <mergeCell ref="A33:B33"/>
     <mergeCell ref="A28:B28"/>
     <mergeCell ref="A32:B32"/>
-    <mergeCell ref="C27:J27"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="A31:B31"/>
-    <mergeCell ref="A34:B34"/>
-    <mergeCell ref="A35:B35"/>
   </mergeCells>
   <conditionalFormatting sqref="A9:P23">
     <cfRule type="expression" dxfId="8" priority="1">
@@ -11965,24 +11983,24 @@
       </c>
     </row>
     <row r="2" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="63" t="s">
+      <c r="A2" s="64" t="s">
         <v>371</v>
       </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="64"/>
-      <c r="D2" s="64"/>
-      <c r="E2" s="64"/>
-      <c r="F2" s="64"/>
-      <c r="G2" s="64"/>
-      <c r="H2" s="64"/>
-      <c r="I2" s="64"/>
-      <c r="J2" s="64"/>
-      <c r="K2" s="64"/>
-      <c r="L2" s="64"/>
-      <c r="M2" s="64"/>
-      <c r="N2" s="64"/>
-      <c r="O2" s="64"/>
-      <c r="P2" s="64"/>
+      <c r="B2" s="65"/>
+      <c r="C2" s="65"/>
+      <c r="D2" s="65"/>
+      <c r="E2" s="65"/>
+      <c r="F2" s="65"/>
+      <c r="G2" s="65"/>
+      <c r="H2" s="65"/>
+      <c r="I2" s="65"/>
+      <c r="J2" s="65"/>
+      <c r="K2" s="65"/>
+      <c r="L2" s="65"/>
+      <c r="M2" s="65"/>
+      <c r="N2" s="65"/>
+      <c r="O2" s="65"/>
+      <c r="P2" s="65"/>
     </row>
     <row r="4" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
@@ -12946,87 +12964,87 @@
       </c>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A22" s="59" t="s">
+      <c r="A22" s="60" t="s">
         <v>383</v>
       </c>
-      <c r="B22" s="62"/>
+      <c r="B22" s="61"/>
       <c r="C22" s="41">
         <f>MAX(K5:K19)</f>
         <v>61.833333333333336</v>
       </c>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A23" s="59" t="s">
+      <c r="A23" s="60" t="s">
         <v>384</v>
       </c>
-      <c r="B23" s="62"/>
-      <c r="C23" s="59" t="str">
+      <c r="B23" s="61"/>
+      <c r="C23" s="60" t="str">
         <f>LEFT(IF(O5="Găng","A → ","")&amp;IF(O6="Găng","B → ","")&amp;IF(O7="Găng","C → ","")&amp;IF(O8="Găng","D → ","")&amp;IF(O9="Găng","E → ","")&amp;IF(O10="Găng","F → ","")&amp;IF(O11="Găng","G → ","")&amp;IF(O12="Găng","H → ","")&amp;IF(O13="Găng","I → ","")&amp;IF(O14="Găng","J → ","")&amp;IF(O15="Găng","K → ","")&amp;IF(O16="Găng","L → ","")&amp;IF(O17="Găng","M → ","")&amp;IF(O18="Găng","N → ","")&amp;IF(O19="Găng","O → ",""),LEN(IF(O5="Găng","A → ","")&amp;IF(O6="Găng","B → ","")&amp;IF(O7="Găng","C → ","")&amp;IF(O8="Găng","D → ","")&amp;IF(O9="Găng","E → ","")&amp;IF(O10="Găng","F → ","")&amp;IF(O11="Găng","G → ","")&amp;IF(O12="Găng","H → ","")&amp;IF(O13="Găng","I → ","")&amp;IF(O14="Găng","J → ","")&amp;IF(O15="Găng","K → ","")&amp;IF(O16="Găng","L → ","")&amp;IF(O17="Găng","M → ","")&amp;IF(O18="Găng","N → ","")&amp;IF(O19="Găng","O → ",""))-3)</f>
         <v>A → B → C → D → F → G → K → M → N → O</v>
       </c>
-      <c r="D23" s="60"/>
-      <c r="E23" s="60"/>
-      <c r="F23" s="60"/>
-      <c r="G23" s="60"/>
-      <c r="H23" s="60"/>
-      <c r="I23" s="60"/>
-      <c r="J23" s="61"/>
+      <c r="D23" s="62"/>
+      <c r="E23" s="62"/>
+      <c r="F23" s="62"/>
+      <c r="G23" s="62"/>
+      <c r="H23" s="62"/>
+      <c r="I23" s="62"/>
+      <c r="J23" s="63"/>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A24" s="59" t="s">
+      <c r="A24" s="60" t="s">
         <v>362</v>
       </c>
-      <c r="B24" s="62"/>
+      <c r="B24" s="61"/>
       <c r="C24" s="41">
         <f>SQRT(SUMIF(O5:O19,"Găng",I5:I19))</f>
         <v>3.3870669054835965</v>
       </c>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A25" s="59" t="s">
+      <c r="A25" s="60" t="s">
         <v>363</v>
       </c>
-      <c r="B25" s="62"/>
+      <c r="B25" s="61"/>
       <c r="C25" s="29">
         <f>PERT!C5</f>
         <v>64</v>
       </c>
     </row>
     <row r="26" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A26" s="59" t="s">
+      <c r="A26" s="60" t="s">
         <v>385</v>
       </c>
-      <c r="B26" s="62"/>
+      <c r="B26" s="61"/>
       <c r="C26" s="41">
         <f>C25-C22</f>
         <v>2.1666666666666643</v>
       </c>
     </row>
     <row r="27" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A27" s="59" t="s">
+      <c r="A27" s="60" t="s">
         <v>386</v>
       </c>
-      <c r="B27" s="62"/>
+      <c r="B27" s="61"/>
       <c r="C27" s="35">
         <f>NORMSDIST((C25-C22)/C24)</f>
         <v>0.73881232950538911</v>
       </c>
     </row>
     <row r="28" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A28" s="59" t="s">
+      <c r="A28" s="60" t="s">
         <v>387</v>
       </c>
-      <c r="B28" s="62"/>
+      <c r="B28" s="61"/>
       <c r="C28" s="43">
         <f>WORKDAY(PERT!C3,ROUNDUP(C22,0)-1)</f>
         <v>46385</v>
       </c>
     </row>
     <row r="29" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A29" s="59" t="s">
+      <c r="A29" s="60" t="s">
         <v>388</v>
       </c>
-      <c r="B29" s="62"/>
+      <c r="B29" s="61"/>
       <c r="C29" s="41">
         <f>PERT!$C$26</f>
         <v>75.333333333333329</v>
@@ -13038,16 +13056,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="C23:J23"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A2:P2"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="A24:B24"/>
     <mergeCell ref="A29:B29"/>
     <mergeCell ref="A25:B25"/>
     <mergeCell ref="A28:B28"/>
     <mergeCell ref="A23:B23"/>
     <mergeCell ref="A27:B27"/>
-    <mergeCell ref="C23:J23"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="A2:P2"/>
-    <mergeCell ref="A26:B26"/>
-    <mergeCell ref="A24:B24"/>
   </mergeCells>
   <conditionalFormatting sqref="A5:O19">
     <cfRule type="expression" dxfId="3" priority="1">
@@ -13341,45 +13359,45 @@
       </c>
     </row>
     <row r="10" spans="1:13" ht="52.8" x14ac:dyDescent="0.3">
-      <c r="A10" s="66" t="s">
+      <c r="A10" s="26" t="s">
         <v>470</v>
       </c>
-      <c r="B10" s="68" t="s">
+      <c r="B10" s="59" t="s">
         <v>479</v>
       </c>
-      <c r="C10" s="68" t="s">
+      <c r="C10" s="59" t="s">
         <v>478</v>
       </c>
-      <c r="D10" s="68" t="s">
+      <c r="D10" s="59" t="s">
         <v>477</v>
       </c>
-      <c r="E10" s="68" t="s">
+      <c r="E10" s="59" t="s">
         <v>436</v>
       </c>
-      <c r="F10" s="67">
+      <c r="F10" s="58">
         <v>3</v>
       </c>
-      <c r="G10" s="67">
+      <c r="G10" s="58">
         <v>4</v>
       </c>
-      <c r="H10" s="67">
+      <c r="H10" s="58">
         <f>IF(OR(F10="",G10=""),"",F10*G10)</f>
         <v>12</v>
       </c>
-      <c r="I10" s="67" t="str">
+      <c r="I10" s="58" t="str">
         <f>IF(H10="","",IF(H10&gt;=15,"Cao",IF(H10&gt;=8,"Trung bình","Thấp")))</f>
         <v>Trung bình</v>
       </c>
-      <c r="J10" s="68" t="s">
+      <c r="J10" s="59" t="s">
         <v>409</v>
       </c>
-      <c r="K10" s="68" t="s">
+      <c r="K10" s="59" t="s">
         <v>480</v>
       </c>
-      <c r="L10" s="68" t="s">
+      <c r="L10" s="59" t="s">
         <v>40</v>
       </c>
-      <c r="M10" s="67" t="s">
+      <c r="M10" s="58" t="s">
         <v>471</v>
       </c>
     </row>
@@ -13512,119 +13530,137 @@
         <v>412</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="52.8" x14ac:dyDescent="0.3">
-      <c r="A14" s="52" t="s">
-        <v>457</v>
-      </c>
-      <c r="B14" s="24" t="s">
-        <v>458</v>
-      </c>
-      <c r="C14" s="24" t="s">
-        <v>459</v>
-      </c>
-      <c r="D14" s="24" t="s">
-        <v>460</v>
-      </c>
-      <c r="E14" s="24" t="s">
-        <v>461</v>
-      </c>
-      <c r="F14" s="53">
-        <v>2</v>
-      </c>
-      <c r="G14" s="53">
-        <v>4</v>
-      </c>
-      <c r="H14" s="54">
-        <f>F14*G14</f>
-        <v>8</v>
-      </c>
-      <c r="I14" s="28" t="str">
-        <f>IF(H14&gt;=15,"Cao",IF(H14&gt;=8,"Trung bình","Thấp"))</f>
+    <row r="14" spans="1:13" ht="66" x14ac:dyDescent="0.3">
+      <c r="A14" s="67" t="s">
+        <v>472</v>
+      </c>
+      <c r="B14" s="69" t="s">
+        <v>484</v>
+      </c>
+      <c r="C14" s="69" t="s">
+        <v>483</v>
+      </c>
+      <c r="D14" s="69" t="s">
+        <v>482</v>
+      </c>
+      <c r="E14" s="69" t="s">
+        <v>481</v>
+      </c>
+      <c r="F14" s="68">
+        <v>3</v>
+      </c>
+      <c r="G14" s="68">
+        <v>3</v>
+      </c>
+      <c r="H14" s="68">
+        <f>IF(OR(F14="",G14=""),"",F14*G14)</f>
+        <v>9</v>
+      </c>
+      <c r="I14" s="68" t="str">
+        <f>IF(H14="","",IF(H14&gt;=15,"Cao",IF(H14&gt;=8,"Trung bình","Thấp")))</f>
         <v>Trung bình</v>
       </c>
-      <c r="J14" s="24" t="s">
+      <c r="J14" s="69" t="s">
         <v>409</v>
       </c>
-      <c r="K14" s="24" t="s">
-        <v>462</v>
-      </c>
-      <c r="L14" s="24" t="s">
+      <c r="K14" s="69" t="s">
+        <v>485</v>
+      </c>
+      <c r="L14" s="69" t="s">
         <v>80</v>
       </c>
-      <c r="M14" s="23" t="s">
-        <v>412</v>
+      <c r="M14" s="68" t="s">
+        <v>471</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="52" t="s">
-        <v>463</v>
+        <v>457</v>
       </c>
       <c r="B15" s="24" t="s">
-        <v>464</v>
+        <v>458</v>
       </c>
       <c r="C15" s="24" t="s">
-        <v>465</v>
+        <v>459</v>
       </c>
       <c r="D15" s="24" t="s">
-        <v>466</v>
+        <v>460</v>
       </c>
       <c r="E15" s="24" t="s">
-        <v>467</v>
+        <v>461</v>
       </c>
       <c r="F15" s="53">
         <v>2</v>
       </c>
       <c r="G15" s="53">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H15" s="54">
         <f>F15*G15</f>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I15" s="28" t="str">
         <f>IF(H15&gt;=15,"Cao",IF(H15&gt;=8,"Trung bình","Thấp"))</f>
-        <v>Thấp</v>
+        <v>Trung bình</v>
       </c>
       <c r="J15" s="24" t="s">
-        <v>468</v>
+        <v>409</v>
       </c>
       <c r="K15" s="24" t="s">
-        <v>469</v>
+        <v>462</v>
       </c>
       <c r="L15" s="24" t="s">
-        <v>105</v>
+        <v>80</v>
       </c>
       <c r="M15" s="23" t="s">
         <v>412</v>
       </c>
     </row>
     <row r="16" spans="1:13" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="26" t="s">
-        <v>472</v>
-      </c>
-      <c r="B16" s="55"/>
-      <c r="C16" s="55"/>
-      <c r="D16" s="55"/>
-      <c r="E16" s="55"/>
-      <c r="F16" s="55"/>
-      <c r="G16" s="55"/>
-      <c r="H16" s="55" t="str">
-        <f>IF(OR(F16="",G16=""),"",F16*G16)</f>
-        <v/>
-      </c>
-      <c r="I16" s="55" t="str">
-        <f>IF(H16="","",IF(H16&gt;=15,"Cao",IF(H16&gt;=8,"Trung bình","Thấp")))</f>
-        <v/>
-      </c>
-      <c r="J16" s="55"/>
-      <c r="K16" s="55"/>
-      <c r="L16" s="55"/>
-      <c r="M16" s="55" t="s">
-        <v>471</v>
+      <c r="A16" s="52" t="s">
+        <v>463</v>
+      </c>
+      <c r="B16" s="24" t="s">
+        <v>464</v>
+      </c>
+      <c r="C16" s="24" t="s">
+        <v>465</v>
+      </c>
+      <c r="D16" s="24" t="s">
+        <v>466</v>
+      </c>
+      <c r="E16" s="24" t="s">
+        <v>467</v>
+      </c>
+      <c r="F16" s="53">
+        <v>2</v>
+      </c>
+      <c r="G16" s="53">
+        <v>3</v>
+      </c>
+      <c r="H16" s="54">
+        <f>F16*G16</f>
+        <v>6</v>
+      </c>
+      <c r="I16" s="28" t="str">
+        <f>IF(H16&gt;=15,"Cao",IF(H16&gt;=8,"Trung bình","Thấp"))</f>
+        <v>Thấp</v>
+      </c>
+      <c r="J16" s="24" t="s">
+        <v>468</v>
+      </c>
+      <c r="K16" s="24" t="s">
+        <v>469</v>
+      </c>
+      <c r="L16" s="24" t="s">
+        <v>105</v>
+      </c>
+      <c r="M16" s="23" t="s">
+        <v>412</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A5:M15">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A5:M16">
     <sortCondition descending="1" ref="H5"/>
   </sortState>
   <conditionalFormatting sqref="I5:I16">
@@ -13658,13 +13694,13 @@
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="C3" s="65" t="s">
+      <c r="C3" s="66" t="s">
         <v>474</v>
       </c>
-      <c r="D3" s="64"/>
-      <c r="E3" s="64"/>
-      <c r="F3" s="64"/>
-      <c r="G3" s="64"/>
+      <c r="D3" s="65"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="65"/>
+      <c r="G3" s="65"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C4" s="7">
@@ -13690,23 +13726,23 @@
       <c r="B5" s="7">
         <v>5</v>
       </c>
-      <c r="C5" s="56" t="str">
+      <c r="C5" s="55" t="str">
         <f>TRIM(IF(AND(RuiRo!$F$5=5,RuiRo!$G$5=1),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=5,RuiRo!$G$6=1),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=5,RuiRo!$G$7=1),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=5,RuiRo!$G$8=1),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=5,RuiRo!$G$9=1),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=5,RuiRo!$G$10=1),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=5,RuiRo!$G$11=1),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=5,RuiRo!$G$12=1),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=5,RuiRo!$G$13=1),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=5,RuiRo!$G$14=1),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=5,RuiRo!$G$15=1),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=5,RuiRo!$G$16=1),RuiRo!$A$16&amp;" ",""))</f>
         <v/>
       </c>
-      <c r="D5" s="57" t="str">
+      <c r="D5" s="56" t="str">
         <f>TRIM(IF(AND(RuiRo!$F$5=5,RuiRo!$G$5=2),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=5,RuiRo!$G$6=2),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=5,RuiRo!$G$7=2),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=5,RuiRo!$G$8=2),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=5,RuiRo!$G$9=2),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=5,RuiRo!$G$10=2),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=5,RuiRo!$G$11=2),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=5,RuiRo!$G$12=2),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=5,RuiRo!$G$13=2),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=5,RuiRo!$G$14=2),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=5,RuiRo!$G$15=2),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=5,RuiRo!$G$16=2),RuiRo!$A$16&amp;" ",""))</f>
         <v/>
       </c>
-      <c r="E5" s="58" t="str">
+      <c r="E5" s="57" t="str">
         <f>TRIM(IF(AND(RuiRo!$F$5=5,RuiRo!$G$5=3),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=5,RuiRo!$G$6=3),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=5,RuiRo!$G$7=3),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=5,RuiRo!$G$8=3),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=5,RuiRo!$G$9=3),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=5,RuiRo!$G$10=3),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=5,RuiRo!$G$11=3),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=5,RuiRo!$G$12=3),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=5,RuiRo!$G$13=3),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=5,RuiRo!$G$14=3),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=5,RuiRo!$G$15=3),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=5,RuiRo!$G$16=3),RuiRo!$A$16&amp;" ",""))</f>
         <v/>
       </c>
-      <c r="F5" s="58" t="str">
+      <c r="F5" s="57" t="str">
         <f>TRIM(IF(AND(RuiRo!$F$5=5,RuiRo!$G$5=4),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=5,RuiRo!$G$6=4),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=5,RuiRo!$G$7=4),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=5,RuiRo!$G$8=4),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=5,RuiRo!$G$9=4),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=5,RuiRo!$G$10=4),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=5,RuiRo!$G$11=4),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=5,RuiRo!$G$12=4),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=5,RuiRo!$G$13=4),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=5,RuiRo!$G$14=4),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=5,RuiRo!$G$15=4),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=5,RuiRo!$G$16=4),RuiRo!$A$16&amp;" ",""))</f>
         <v/>
       </c>
-      <c r="G5" s="58" t="str">
+      <c r="G5" s="57" t="str">
         <f>TRIM(IF(AND(RuiRo!$F$5=5,RuiRo!$G$5=5),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=5,RuiRo!$G$6=5),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=5,RuiRo!$G$7=5),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=5,RuiRo!$G$8=5),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=5,RuiRo!$G$9=5),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=5,RuiRo!$G$10=5),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=5,RuiRo!$G$11=5),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=5,RuiRo!$G$12=5),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=5,RuiRo!$G$13=5),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=5,RuiRo!$G$14=5),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=5,RuiRo!$G$15=5),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=5,RuiRo!$G$16=5),RuiRo!$A$16&amp;" ",""))</f>
         <v/>
       </c>
@@ -13715,23 +13751,23 @@
       <c r="B6" s="7">
         <v>4</v>
       </c>
-      <c r="C6" s="56" t="str">
+      <c r="C6" s="55" t="str">
         <f>TRIM(IF(AND(RuiRo!$F$5=4,RuiRo!$G$5=1),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=4,RuiRo!$G$6=1),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=4,RuiRo!$G$7=1),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=4,RuiRo!$G$8=1),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=4,RuiRo!$G$9=1),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=4,RuiRo!$G$10=1),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=4,RuiRo!$G$11=1),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=4,RuiRo!$G$12=1),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=4,RuiRo!$G$13=1),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=4,RuiRo!$G$14=1),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=4,RuiRo!$G$15=1),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=4,RuiRo!$G$16=1),RuiRo!$A$16&amp;" ",""))</f>
         <v/>
       </c>
-      <c r="D6" s="57" t="str">
+      <c r="D6" s="56" t="str">
         <f>TRIM(IF(AND(RuiRo!$F$5=4,RuiRo!$G$5=2),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=4,RuiRo!$G$6=2),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=4,RuiRo!$G$7=2),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=4,RuiRo!$G$8=2),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=4,RuiRo!$G$9=2),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=4,RuiRo!$G$10=2),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=4,RuiRo!$G$11=2),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=4,RuiRo!$G$12=2),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=4,RuiRo!$G$13=2),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=4,RuiRo!$G$14=2),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=4,RuiRo!$G$15=2),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=4,RuiRo!$G$16=2),RuiRo!$A$16&amp;" ",""))</f>
         <v/>
       </c>
-      <c r="E6" s="57" t="str">
+      <c r="E6" s="56" t="str">
         <f>TRIM(IF(AND(RuiRo!$F$5=4,RuiRo!$G$5=3),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=4,RuiRo!$G$6=3),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=4,RuiRo!$G$7=3),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=4,RuiRo!$G$8=3),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=4,RuiRo!$G$9=3),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=4,RuiRo!$G$10=3),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=4,RuiRo!$G$11=3),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=4,RuiRo!$G$12=3),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=4,RuiRo!$G$13=3),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=4,RuiRo!$G$14=3),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=4,RuiRo!$G$15=3),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=4,RuiRo!$G$16=3),RuiRo!$A$16&amp;" ",""))</f>
         <v/>
       </c>
-      <c r="F6" s="58" t="str">
+      <c r="F6" s="57" t="str">
         <f>TRIM(IF(AND(RuiRo!$F$5=4,RuiRo!$G$5=4),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=4,RuiRo!$G$6=4),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=4,RuiRo!$G$7=4),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=4,RuiRo!$G$8=4),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=4,RuiRo!$G$9=4),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=4,RuiRo!$G$10=4),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=4,RuiRo!$G$11=4),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=4,RuiRo!$G$12=4),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=4,RuiRo!$G$13=4),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=4,RuiRo!$G$14=4),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=4,RuiRo!$G$15=4),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=4,RuiRo!$G$16=4),RuiRo!$A$16&amp;" ",""))</f>
         <v>R02 R03 R04</v>
       </c>
-      <c r="G6" s="58" t="str">
+      <c r="G6" s="57" t="str">
         <f>TRIM(IF(AND(RuiRo!$F$5=4,RuiRo!$G$5=5),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=4,RuiRo!$G$6=5),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=4,RuiRo!$G$7=5),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=4,RuiRo!$G$8=5),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=4,RuiRo!$G$9=5),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=4,RuiRo!$G$10=5),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=4,RuiRo!$G$11=5),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=4,RuiRo!$G$12=5),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=4,RuiRo!$G$13=5),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=4,RuiRo!$G$14=5),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=4,RuiRo!$G$15=5),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=4,RuiRo!$G$16=5),RuiRo!$A$16&amp;" ",""))</f>
         <v>R01</v>
       </c>
@@ -13740,23 +13776,23 @@
       <c r="B7" s="7">
         <v>3</v>
       </c>
-      <c r="C7" s="56" t="str">
+      <c r="C7" s="55" t="str">
         <f>TRIM(IF(AND(RuiRo!$F$5=3,RuiRo!$G$5=1),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=3,RuiRo!$G$6=1),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=3,RuiRo!$G$7=1),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=3,RuiRo!$G$8=1),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=3,RuiRo!$G$9=1),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=3,RuiRo!$G$10=1),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=3,RuiRo!$G$11=1),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=3,RuiRo!$G$12=1),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=3,RuiRo!$G$13=1),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=3,RuiRo!$G$14=1),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=3,RuiRo!$G$15=1),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=3,RuiRo!$G$16=1),RuiRo!$A$16&amp;" ",""))</f>
         <v/>
       </c>
-      <c r="D7" s="56" t="str">
+      <c r="D7" s="55" t="str">
         <f>TRIM(IF(AND(RuiRo!$F$5=3,RuiRo!$G$5=2),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=3,RuiRo!$G$6=2),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=3,RuiRo!$G$7=2),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=3,RuiRo!$G$8=2),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=3,RuiRo!$G$9=2),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=3,RuiRo!$G$10=2),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=3,RuiRo!$G$11=2),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=3,RuiRo!$G$12=2),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=3,RuiRo!$G$13=2),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=3,RuiRo!$G$14=2),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=3,RuiRo!$G$15=2),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=3,RuiRo!$G$16=2),RuiRo!$A$16&amp;" ",""))</f>
         <v/>
       </c>
-      <c r="E7" s="57" t="str">
+      <c r="E7" s="56" t="str">
         <f>TRIM(IF(AND(RuiRo!$F$5=3,RuiRo!$G$5=3),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=3,RuiRo!$G$6=3),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=3,RuiRo!$G$7=3),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=3,RuiRo!$G$8=3),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=3,RuiRo!$G$9=3),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=3,RuiRo!$G$10=3),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=3,RuiRo!$G$11=3),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=3,RuiRo!$G$12=3),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=3,RuiRo!$G$13=3),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=3,RuiRo!$G$14=3),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=3,RuiRo!$G$15=3),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=3,RuiRo!$G$16=3),RuiRo!$A$16&amp;" ",""))</f>
-        <v>R07 R08</v>
-      </c>
-      <c r="F7" s="57" t="str">
+        <v>R07 R08 R12</v>
+      </c>
+      <c r="F7" s="56" t="str">
         <f>TRIM(IF(AND(RuiRo!$F$5=3,RuiRo!$G$5=4),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=3,RuiRo!$G$6=4),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=3,RuiRo!$G$7=4),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=3,RuiRo!$G$8=4),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=3,RuiRo!$G$9=4),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=3,RuiRo!$G$10=4),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=3,RuiRo!$G$11=4),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=3,RuiRo!$G$12=4),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=3,RuiRo!$G$13=4),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=3,RuiRo!$G$14=4),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=3,RuiRo!$G$15=4),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=3,RuiRo!$G$16=4),RuiRo!$A$16&amp;" ",""))</f>
         <v>R11</v>
       </c>
-      <c r="G7" s="58" t="str">
+      <c r="G7" s="57" t="str">
         <f>TRIM(IF(AND(RuiRo!$F$5=3,RuiRo!$G$5=5),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=3,RuiRo!$G$6=5),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=3,RuiRo!$G$7=5),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=3,RuiRo!$G$8=5),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=3,RuiRo!$G$9=5),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=3,RuiRo!$G$10=5),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=3,RuiRo!$G$11=5),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=3,RuiRo!$G$12=5),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=3,RuiRo!$G$13=5),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=3,RuiRo!$G$14=5),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=3,RuiRo!$G$15=5),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=3,RuiRo!$G$16=5),RuiRo!$A$16&amp;" ",""))</f>
         <v>R05</v>
       </c>
@@ -13765,23 +13801,23 @@
       <c r="B8" s="7">
         <v>2</v>
       </c>
-      <c r="C8" s="56" t="str">
+      <c r="C8" s="55" t="str">
         <f>TRIM(IF(AND(RuiRo!$F$5=2,RuiRo!$G$5=1),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=2,RuiRo!$G$6=1),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=2,RuiRo!$G$7=1),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=2,RuiRo!$G$8=1),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=2,RuiRo!$G$9=1),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=2,RuiRo!$G$10=1),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=2,RuiRo!$G$11=1),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=2,RuiRo!$G$12=1),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=2,RuiRo!$G$13=1),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=2,RuiRo!$G$14=1),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=2,RuiRo!$G$15=1),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=2,RuiRo!$G$16=1),RuiRo!$A$16&amp;" ",""))</f>
         <v/>
       </c>
-      <c r="D8" s="56" t="str">
+      <c r="D8" s="55" t="str">
         <f>TRIM(IF(AND(RuiRo!$F$5=2,RuiRo!$G$5=2),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=2,RuiRo!$G$6=2),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=2,RuiRo!$G$7=2),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=2,RuiRo!$G$8=2),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=2,RuiRo!$G$9=2),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=2,RuiRo!$G$10=2),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=2,RuiRo!$G$11=2),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=2,RuiRo!$G$12=2),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=2,RuiRo!$G$13=2),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=2,RuiRo!$G$14=2),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=2,RuiRo!$G$15=2),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=2,RuiRo!$G$16=2),RuiRo!$A$16&amp;" ",""))</f>
         <v/>
       </c>
-      <c r="E8" s="56" t="str">
+      <c r="E8" s="55" t="str">
         <f>TRIM(IF(AND(RuiRo!$F$5=2,RuiRo!$G$5=3),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=2,RuiRo!$G$6=3),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=2,RuiRo!$G$7=3),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=2,RuiRo!$G$8=3),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=2,RuiRo!$G$9=3),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=2,RuiRo!$G$10=3),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=2,RuiRo!$G$11=3),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=2,RuiRo!$G$12=3),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=2,RuiRo!$G$13=3),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=2,RuiRo!$G$14=3),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=2,RuiRo!$G$15=3),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=2,RuiRo!$G$16=3),RuiRo!$A$16&amp;" ",""))</f>
         <v>R10</v>
       </c>
-      <c r="F8" s="57" t="str">
+      <c r="F8" s="56" t="str">
         <f>TRIM(IF(AND(RuiRo!$F$5=2,RuiRo!$G$5=4),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=2,RuiRo!$G$6=4),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=2,RuiRo!$G$7=4),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=2,RuiRo!$G$8=4),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=2,RuiRo!$G$9=4),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=2,RuiRo!$G$10=4),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=2,RuiRo!$G$11=4),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=2,RuiRo!$G$12=4),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=2,RuiRo!$G$13=4),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=2,RuiRo!$G$14=4),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=2,RuiRo!$G$15=4),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=2,RuiRo!$G$16=4),RuiRo!$A$16&amp;" ",""))</f>
         <v>R09</v>
       </c>
-      <c r="G8" s="57" t="str">
+      <c r="G8" s="56" t="str">
         <f>TRIM(IF(AND(RuiRo!$F$5=2,RuiRo!$G$5=5),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=2,RuiRo!$G$6=5),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=2,RuiRo!$G$7=5),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=2,RuiRo!$G$8=5),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=2,RuiRo!$G$9=5),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=2,RuiRo!$G$10=5),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=2,RuiRo!$G$11=5),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=2,RuiRo!$G$12=5),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=2,RuiRo!$G$13=5),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=2,RuiRo!$G$14=5),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=2,RuiRo!$G$15=5),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=2,RuiRo!$G$16=5),RuiRo!$A$16&amp;" ",""))</f>
         <v>R06</v>
       </c>
@@ -13790,23 +13826,23 @@
       <c r="B9" s="7">
         <v>1</v>
       </c>
-      <c r="C9" s="56" t="str">
+      <c r="C9" s="55" t="str">
         <f>TRIM(IF(AND(RuiRo!$F$5=1,RuiRo!$G$5=1),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=1,RuiRo!$G$6=1),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=1,RuiRo!$G$7=1),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=1,RuiRo!$G$8=1),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=1,RuiRo!$G$9=1),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=1,RuiRo!$G$10=1),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=1,RuiRo!$G$11=1),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=1,RuiRo!$G$12=1),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=1,RuiRo!$G$13=1),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=1,RuiRo!$G$14=1),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=1,RuiRo!$G$15=1),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=1,RuiRo!$G$16=1),RuiRo!$A$16&amp;" ",""))</f>
         <v/>
       </c>
-      <c r="D9" s="56" t="str">
+      <c r="D9" s="55" t="str">
         <f>TRIM(IF(AND(RuiRo!$F$5=1,RuiRo!$G$5=2),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=1,RuiRo!$G$6=2),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=1,RuiRo!$G$7=2),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=1,RuiRo!$G$8=2),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=1,RuiRo!$G$9=2),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=1,RuiRo!$G$10=2),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=1,RuiRo!$G$11=2),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=1,RuiRo!$G$12=2),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=1,RuiRo!$G$13=2),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=1,RuiRo!$G$14=2),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=1,RuiRo!$G$15=2),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=1,RuiRo!$G$16=2),RuiRo!$A$16&amp;" ",""))</f>
         <v/>
       </c>
-      <c r="E9" s="56" t="str">
+      <c r="E9" s="55" t="str">
         <f>TRIM(IF(AND(RuiRo!$F$5=1,RuiRo!$G$5=3),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=1,RuiRo!$G$6=3),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=1,RuiRo!$G$7=3),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=1,RuiRo!$G$8=3),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=1,RuiRo!$G$9=3),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=1,RuiRo!$G$10=3),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=1,RuiRo!$G$11=3),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=1,RuiRo!$G$12=3),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=1,RuiRo!$G$13=3),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=1,RuiRo!$G$14=3),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=1,RuiRo!$G$15=3),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=1,RuiRo!$G$16=3),RuiRo!$A$16&amp;" ",""))</f>
         <v/>
       </c>
-      <c r="F9" s="56" t="str">
+      <c r="F9" s="55" t="str">
         <f>TRIM(IF(AND(RuiRo!$F$5=1,RuiRo!$G$5=4),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=1,RuiRo!$G$6=4),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=1,RuiRo!$G$7=4),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=1,RuiRo!$G$8=4),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=1,RuiRo!$G$9=4),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=1,RuiRo!$G$10=4),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=1,RuiRo!$G$11=4),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=1,RuiRo!$G$12=4),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=1,RuiRo!$G$13=4),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=1,RuiRo!$G$14=4),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=1,RuiRo!$G$15=4),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=1,RuiRo!$G$16=4),RuiRo!$A$16&amp;" ",""))</f>
         <v/>
       </c>
-      <c r="G9" s="56" t="str">
+      <c r="G9" s="55" t="str">
         <f>TRIM(IF(AND(RuiRo!$F$5=1,RuiRo!$G$5=5),RuiRo!$A$5&amp;" ","")&amp;IF(AND(RuiRo!$F$6=1,RuiRo!$G$6=5),RuiRo!$A$6&amp;" ","")&amp;IF(AND(RuiRo!$F$7=1,RuiRo!$G$7=5),RuiRo!$A$7&amp;" ","")&amp;IF(AND(RuiRo!$F$8=1,RuiRo!$G$8=5),RuiRo!$A$8&amp;" ","")&amp;IF(AND(RuiRo!$F$9=1,RuiRo!$G$9=5),RuiRo!$A$9&amp;" ","")&amp;IF(AND(RuiRo!$F$10=1,RuiRo!$G$10=5),RuiRo!$A$10&amp;" ","")&amp;IF(AND(RuiRo!$F$11=1,RuiRo!$G$11=5),RuiRo!$A$11&amp;" ","")&amp;IF(AND(RuiRo!$F$12=1,RuiRo!$G$12=5),RuiRo!$A$12&amp;" ","")&amp;IF(AND(RuiRo!$F$13=1,RuiRo!$G$13=5),RuiRo!$A$13&amp;" ","")&amp;IF(AND(RuiRo!$F$14=1,RuiRo!$G$14=5),RuiRo!$A$14&amp;" ","")&amp;IF(AND(RuiRo!$F$15=1,RuiRo!$G$15=5),RuiRo!$A$15&amp;" ","")&amp;IF(AND(RuiRo!$F$16=1,RuiRo!$G$16=5),RuiRo!$A$16&amp;" ",""))</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Báo cáo lab: thêm phụ lục minh chứng (danh mục, lịch sử commit, ảnh web app, bảng phân công)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/lab/QLDA_PharmaDash_LichDuAn.xlsx
+++ b/docs/lab/QLDA_PharmaDash_LichDuAn.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\nhà thuốc\docs\lab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C3AE40B-9E93-43A1-A886-E7437CB23D77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFECE5D9-2D0E-4B86-BE36-E524E50C04B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="HuongDan" sheetId="1" r:id="rId1"/>
@@ -1718,7 +1718,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1826,22 +1826,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -5723,7 +5716,7 @@
       <c r="A26" s="60" t="s">
         <v>359</v>
       </c>
-      <c r="B26" s="61"/>
+      <c r="B26" s="63"/>
       <c r="C26" s="41">
         <f>MAX(L9:L23)</f>
         <v>75.333333333333329</v>
@@ -5733,24 +5726,24 @@
       <c r="A27" s="60" t="s">
         <v>360</v>
       </c>
-      <c r="B27" s="61"/>
+      <c r="B27" s="63"/>
       <c r="C27" s="60" t="str">
         <f>LEFT(IF(P9="Găng","A → ","")&amp;IF(P10="Găng","B → ","")&amp;IF(P11="Găng","C → ","")&amp;IF(P12="Găng","D → ","")&amp;IF(P13="Găng","E → ","")&amp;IF(P14="Găng","F → ","")&amp;IF(P15="Găng","G → ","")&amp;IF(P16="Găng","H → ","")&amp;IF(P17="Găng","I → ","")&amp;IF(P18="Găng","J → ","")&amp;IF(P19="Găng","K → ","")&amp;IF(P20="Găng","L → ","")&amp;IF(P21="Găng","M → ","")&amp;IF(P22="Găng","N → ","")&amp;IF(P23="Găng","O → ",""),LEN(IF(P9="Găng","A → ","")&amp;IF(P10="Găng","B → ","")&amp;IF(P11="Găng","C → ","")&amp;IF(P12="Găng","D → ","")&amp;IF(P13="Găng","E → ","")&amp;IF(P14="Găng","F → ","")&amp;IF(P15="Găng","G → ","")&amp;IF(P16="Găng","H → ","")&amp;IF(P17="Găng","I → ","")&amp;IF(P18="Găng","J → ","")&amp;IF(P19="Găng","K → ","")&amp;IF(P20="Găng","L → ","")&amp;IF(P21="Găng","M → ","")&amp;IF(P22="Găng","N → ","")&amp;IF(P23="Găng","O → ",""))-3)</f>
         <v>A → B → C → E → I → J → M → N → O</v>
       </c>
-      <c r="D27" s="62"/>
-      <c r="E27" s="62"/>
-      <c r="F27" s="62"/>
-      <c r="G27" s="62"/>
-      <c r="H27" s="62"/>
-      <c r="I27" s="62"/>
-      <c r="J27" s="63"/>
+      <c r="D27" s="61"/>
+      <c r="E27" s="61"/>
+      <c r="F27" s="61"/>
+      <c r="G27" s="61"/>
+      <c r="H27" s="61"/>
+      <c r="I27" s="61"/>
+      <c r="J27" s="62"/>
     </row>
     <row r="28" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A28" s="60" t="s">
         <v>361</v>
       </c>
-      <c r="B28" s="61"/>
+      <c r="B28" s="63"/>
       <c r="C28" s="41">
         <f>SUMIF(P9:P23,"Găng",J9:J23)</f>
         <v>13.055555555555557</v>
@@ -5760,7 +5753,7 @@
       <c r="A29" s="60" t="s">
         <v>362</v>
       </c>
-      <c r="B29" s="61"/>
+      <c r="B29" s="63"/>
       <c r="C29" s="41">
         <f>SQRT(C28)</f>
         <v>3.6132472314464668</v>
@@ -5770,7 +5763,7 @@
       <c r="A30" s="60" t="s">
         <v>363</v>
       </c>
-      <c r="B30" s="61"/>
+      <c r="B30" s="63"/>
       <c r="C30" s="29">
         <f>C5</f>
         <v>64</v>
@@ -5780,7 +5773,7 @@
       <c r="A31" s="60" t="s">
         <v>364</v>
       </c>
-      <c r="B31" s="61"/>
+      <c r="B31" s="63"/>
       <c r="C31" s="41">
         <f>C26-C30</f>
         <v>11.333333333333329</v>
@@ -5790,7 +5783,7 @@
       <c r="A32" s="60" t="s">
         <v>365</v>
       </c>
-      <c r="B32" s="61"/>
+      <c r="B32" s="63"/>
       <c r="C32" s="41">
         <f>(C30-C26)/C29</f>
         <v>-3.1366061072982077</v>
@@ -5800,7 +5793,7 @@
       <c r="A33" s="60" t="s">
         <v>366</v>
       </c>
-      <c r="B33" s="61"/>
+      <c r="B33" s="63"/>
       <c r="C33" s="42">
         <f>NORMSDIST(C32)</f>
         <v>8.5457789242917941E-4</v>
@@ -5810,7 +5803,7 @@
       <c r="A34" s="60" t="s">
         <v>367</v>
       </c>
-      <c r="B34" s="61"/>
+      <c r="B34" s="63"/>
       <c r="C34" s="43">
         <f>WORKDAY(C3,ROUNDUP(C26,0)-1)</f>
         <v>46405</v>
@@ -5820,7 +5813,7 @@
       <c r="A35" s="60" t="s">
         <v>298</v>
       </c>
-      <c r="B35" s="61"/>
+      <c r="B35" s="63"/>
       <c r="C35" s="26" t="str">
         <f>IF(C31&lt;=0,"Kịp hạn chót","TRỄ HẠN – cần nén lịch (crashing / fast-tracking)")</f>
         <v>TRỄ HẠN – cần nén lịch (crashing / fast-tracking)</v>
@@ -5828,17 +5821,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="C27:J27"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="A31:B31"/>
-    <mergeCell ref="A34:B34"/>
-    <mergeCell ref="A35:B35"/>
     <mergeCell ref="A26:B26"/>
     <mergeCell ref="A30:B30"/>
     <mergeCell ref="A29:B29"/>
     <mergeCell ref="A33:B33"/>
     <mergeCell ref="A28:B28"/>
     <mergeCell ref="A32:B32"/>
+    <mergeCell ref="C27:J27"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="A35:B35"/>
   </mergeCells>
   <conditionalFormatting sqref="A9:P23">
     <cfRule type="expression" dxfId="8" priority="1">
@@ -12967,7 +12960,7 @@
       <c r="A22" s="60" t="s">
         <v>383</v>
       </c>
-      <c r="B22" s="61"/>
+      <c r="B22" s="63"/>
       <c r="C22" s="41">
         <f>MAX(K5:K19)</f>
         <v>61.833333333333336</v>
@@ -12977,24 +12970,24 @@
       <c r="A23" s="60" t="s">
         <v>384</v>
       </c>
-      <c r="B23" s="61"/>
+      <c r="B23" s="63"/>
       <c r="C23" s="60" t="str">
         <f>LEFT(IF(O5="Găng","A → ","")&amp;IF(O6="Găng","B → ","")&amp;IF(O7="Găng","C → ","")&amp;IF(O8="Găng","D → ","")&amp;IF(O9="Găng","E → ","")&amp;IF(O10="Găng","F → ","")&amp;IF(O11="Găng","G → ","")&amp;IF(O12="Găng","H → ","")&amp;IF(O13="Găng","I → ","")&amp;IF(O14="Găng","J → ","")&amp;IF(O15="Găng","K → ","")&amp;IF(O16="Găng","L → ","")&amp;IF(O17="Găng","M → ","")&amp;IF(O18="Găng","N → ","")&amp;IF(O19="Găng","O → ",""),LEN(IF(O5="Găng","A → ","")&amp;IF(O6="Găng","B → ","")&amp;IF(O7="Găng","C → ","")&amp;IF(O8="Găng","D → ","")&amp;IF(O9="Găng","E → ","")&amp;IF(O10="Găng","F → ","")&amp;IF(O11="Găng","G → ","")&amp;IF(O12="Găng","H → ","")&amp;IF(O13="Găng","I → ","")&amp;IF(O14="Găng","J → ","")&amp;IF(O15="Găng","K → ","")&amp;IF(O16="Găng","L → ","")&amp;IF(O17="Găng","M → ","")&amp;IF(O18="Găng","N → ","")&amp;IF(O19="Găng","O → ",""))-3)</f>
         <v>A → B → C → D → F → G → K → M → N → O</v>
       </c>
-      <c r="D23" s="62"/>
-      <c r="E23" s="62"/>
-      <c r="F23" s="62"/>
-      <c r="G23" s="62"/>
-      <c r="H23" s="62"/>
-      <c r="I23" s="62"/>
-      <c r="J23" s="63"/>
+      <c r="D23" s="61"/>
+      <c r="E23" s="61"/>
+      <c r="F23" s="61"/>
+      <c r="G23" s="61"/>
+      <c r="H23" s="61"/>
+      <c r="I23" s="61"/>
+      <c r="J23" s="62"/>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A24" s="60" t="s">
         <v>362</v>
       </c>
-      <c r="B24" s="61"/>
+      <c r="B24" s="63"/>
       <c r="C24" s="41">
         <f>SQRT(SUMIF(O5:O19,"Găng",I5:I19))</f>
         <v>3.3870669054835965</v>
@@ -13004,7 +12997,7 @@
       <c r="A25" s="60" t="s">
         <v>363</v>
       </c>
-      <c r="B25" s="61"/>
+      <c r="B25" s="63"/>
       <c r="C25" s="29">
         <f>PERT!C5</f>
         <v>64</v>
@@ -13014,7 +13007,7 @@
       <c r="A26" s="60" t="s">
         <v>385</v>
       </c>
-      <c r="B26" s="61"/>
+      <c r="B26" s="63"/>
       <c r="C26" s="41">
         <f>C25-C22</f>
         <v>2.1666666666666643</v>
@@ -13024,7 +13017,7 @@
       <c r="A27" s="60" t="s">
         <v>386</v>
       </c>
-      <c r="B27" s="61"/>
+      <c r="B27" s="63"/>
       <c r="C27" s="35">
         <f>NORMSDIST((C25-C22)/C24)</f>
         <v>0.73881232950538911</v>
@@ -13034,7 +13027,7 @@
       <c r="A28" s="60" t="s">
         <v>387</v>
       </c>
-      <c r="B28" s="61"/>
+      <c r="B28" s="63"/>
       <c r="C28" s="43">
         <f>WORKDAY(PERT!C3,ROUNDUP(C22,0)-1)</f>
         <v>46385</v>
@@ -13044,7 +13037,7 @@
       <c r="A29" s="60" t="s">
         <v>388</v>
       </c>
-      <c r="B29" s="61"/>
+      <c r="B29" s="63"/>
       <c r="C29" s="41">
         <f>PERT!$C$26</f>
         <v>75.333333333333329</v>
@@ -13056,16 +13049,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A27:B27"/>
     <mergeCell ref="C23:J23"/>
     <mergeCell ref="A22:B22"/>
     <mergeCell ref="A2:P2"/>
     <mergeCell ref="A26:B26"/>
     <mergeCell ref="A24:B24"/>
-    <mergeCell ref="A29:B29"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="A27:B27"/>
   </mergeCells>
   <conditionalFormatting sqref="A5:O19">
     <cfRule type="expression" dxfId="3" priority="1">
@@ -13531,45 +13524,45 @@
       </c>
     </row>
     <row r="14" spans="1:13" ht="66" x14ac:dyDescent="0.3">
-      <c r="A14" s="67" t="s">
+      <c r="A14" s="26" t="s">
         <v>472</v>
       </c>
-      <c r="B14" s="69" t="s">
+      <c r="B14" s="59" t="s">
         <v>484</v>
       </c>
-      <c r="C14" s="69" t="s">
+      <c r="C14" s="59" t="s">
         <v>483</v>
       </c>
-      <c r="D14" s="69" t="s">
+      <c r="D14" s="59" t="s">
         <v>482</v>
       </c>
-      <c r="E14" s="69" t="s">
+      <c r="E14" s="59" t="s">
         <v>481</v>
       </c>
-      <c r="F14" s="68">
+      <c r="F14" s="58">
         <v>3</v>
       </c>
-      <c r="G14" s="68">
+      <c r="G14" s="58">
         <v>3</v>
       </c>
-      <c r="H14" s="68">
+      <c r="H14" s="58">
         <f>IF(OR(F14="",G14=""),"",F14*G14)</f>
         <v>9</v>
       </c>
-      <c r="I14" s="68" t="str">
+      <c r="I14" s="58" t="str">
         <f>IF(H14="","",IF(H14&gt;=15,"Cao",IF(H14&gt;=8,"Trung bình","Thấp")))</f>
         <v>Trung bình</v>
       </c>
-      <c r="J14" s="69" t="s">
+      <c r="J14" s="59" t="s">
         <v>409</v>
       </c>
-      <c r="K14" s="69" t="s">
+      <c r="K14" s="59" t="s">
         <v>485</v>
       </c>
-      <c r="L14" s="69" t="s">
+      <c r="L14" s="59" t="s">
         <v>80</v>
       </c>
-      <c r="M14" s="68" t="s">
+      <c r="M14" s="58" t="s">
         <v>471</v>
       </c>
     </row>

</xml_diff>